<commit_message>
doc(work logs) : updating
</commit_message>
<xml_diff>
--- a/T_CraftMeUp_NeoDarbellay.xlsx
+++ b/T_CraftMeUp_NeoDarbellay.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01Modules\02Deuxieme_Annee\P_Prod\CraftMeUp\Craft-Me-Up\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A7A51EA-2641-485E-B2ED-30FBC6DDA677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1561886-3A06-49C1-84E4-F67D31D00C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Restrictions" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$G$109</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$G$106</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="155">
   <si>
     <t>Experts </t>
   </si>
@@ -495,6 +495,18 @@
   <si>
     <t>Reduced rendering lag as much as I could for today
 You can now start the game with 128x128 chunks, but it is incredibly laggy</t>
+  </si>
+  <si>
+    <t>Optimized the code even more</t>
+  </si>
+  <si>
+    <t>Made it so that after a certain level of zoom, obstacles turn into solid color images and used a few code shortcuts to make it way cleaner</t>
+  </si>
+  <si>
+    <t>More optimization</t>
+  </si>
+  <si>
+    <t>Tried to get rid of "TextHelpers", but it ended up creating more issues than anything. Next step is to cache</t>
   </si>
 </sst>
 </file>
@@ -820,26 +832,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -853,24 +854,35 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="83">
+  <dxfs count="85">
     <dxf>
       <fill>
         <patternFill>
@@ -1175,6 +1187,27 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
@@ -1182,6 +1215,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -1189,6 +1229,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -1224,6 +1271,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -1231,6 +1285,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
@@ -1245,6 +1306,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
@@ -1252,6 +1320,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -1259,6 +1334,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -1280,6 +1362,20 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
@@ -1287,6 +1383,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -1294,6 +1397,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -1301,6 +1411,20 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -1308,6 +1432,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
@@ -1315,6 +1446,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -1322,119 +1460,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1762,7 +1788,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G111"/>
+  <dimension ref="A1:G108"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -1780,65 +1806,65 @@
       <c r="A1" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="35"/>
-      <c r="D1" s="38" t="s">
+      <c r="C1" s="38"/>
+      <c r="D1" s="35" t="s">
         <v>86</v>
       </c>
-      <c r="E1" s="39"/>
-      <c r="F1" s="36" t="s">
+      <c r="E1" s="36"/>
+      <c r="F1" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="37"/>
+      <c r="G1" s="34"/>
     </row>
     <row r="2" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="35"/>
-      <c r="D2" s="38" t="s">
+      <c r="C2" s="38"/>
+      <c r="D2" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="36" t="s">
+      <c r="E2" s="36"/>
+      <c r="F2" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="37"/>
+      <c r="G2" s="34"/>
     </row>
     <row r="3" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="39" t="s">
         <v>129</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="38" t="s">
+      <c r="C3" s="40"/>
+      <c r="D3" s="35" t="s">
         <v>87</v>
       </c>
-      <c r="E3" s="39"/>
-      <c r="F3" s="33" t="s">
+      <c r="E3" s="36"/>
+      <c r="F3" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="35"/>
+      <c r="G3" s="38"/>
     </row>
     <row r="4" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="35"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="38"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1936,13 +1962,13 @@
       <c r="C9" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D9" s="31">
+      <c r="D9" s="41">
         <f>SUM(C6:C8)</f>
         <v>125</v>
       </c>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="32"/>
+      <c r="E9" s="41"/>
+      <c r="F9" s="41"/>
+      <c r="G9" s="42"/>
     </row>
     <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
@@ -2030,7 +2056,7 @@
       <c r="A14" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="30"/>
+      <c r="B14" s="32"/>
       <c r="C14" s="9">
         <v>35</v>
       </c>
@@ -2057,13 +2083,13 @@
       <c r="C15" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D15" s="31">
+      <c r="D15" s="41">
         <f>SUM(C10:C14)</f>
         <v>175</v>
       </c>
-      <c r="E15" s="31"/>
-      <c r="F15" s="31"/>
-      <c r="G15" s="32"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="41"/>
+      <c r="G15" s="42"/>
     </row>
     <row r="16" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
@@ -2140,13 +2166,13 @@
       <c r="C19" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D19" s="31">
+      <c r="D19" s="41">
         <f>SUM(C16:C18)</f>
         <v>145</v>
       </c>
-      <c r="E19" s="31"/>
-      <c r="F19" s="31"/>
-      <c r="G19" s="32"/>
+      <c r="E19" s="41"/>
+      <c r="F19" s="41"/>
+      <c r="G19" s="42"/>
     </row>
     <row r="20" spans="1:7" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
@@ -2200,13 +2226,13 @@
       <c r="C22" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D22" s="31">
+      <c r="D22" s="41">
         <f>SUM(C20:C21)</f>
         <v>105</v>
       </c>
-      <c r="E22" s="31"/>
-      <c r="F22" s="31"/>
-      <c r="G22" s="32"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="42"/>
     </row>
     <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
@@ -2281,13 +2307,13 @@
       <c r="C26" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D26" s="31">
+      <c r="D26" s="41">
         <f>SUM(C23:C25)</f>
         <v>140</v>
       </c>
-      <c r="E26" s="31"/>
-      <c r="F26" s="31"/>
-      <c r="G26" s="32"/>
+      <c r="E26" s="41"/>
+      <c r="F26" s="41"/>
+      <c r="G26" s="42"/>
     </row>
     <row r="27" spans="1:7" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
@@ -2362,13 +2388,13 @@
       <c r="C30" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D30" s="31">
+      <c r="D30" s="41">
         <f>SUM(C27:C29)</f>
         <v>155</v>
       </c>
-      <c r="E30" s="31"/>
-      <c r="F30" s="31"/>
-      <c r="G30" s="32"/>
+      <c r="E30" s="41"/>
+      <c r="F30" s="41"/>
+      <c r="G30" s="42"/>
     </row>
     <row r="31" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
@@ -2557,13 +2583,13 @@
       <c r="C40" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D40" s="31">
+      <c r="D40" s="41">
         <f>SUM(C31:C39)</f>
         <v>140</v>
       </c>
-      <c r="E40" s="31"/>
-      <c r="F40" s="31"/>
-      <c r="G40" s="32"/>
+      <c r="E40" s="41"/>
+      <c r="F40" s="41"/>
+      <c r="G40" s="42"/>
     </row>
     <row r="41" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
@@ -2617,13 +2643,13 @@
       <c r="C43" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D43" s="31">
+      <c r="D43" s="41">
         <f>SUM(C41:C42)</f>
         <v>190</v>
       </c>
-      <c r="E43" s="31"/>
-      <c r="F43" s="31"/>
-      <c r="G43" s="32"/>
+      <c r="E43" s="41"/>
+      <c r="F43" s="41"/>
+      <c r="G43" s="42"/>
     </row>
     <row r="44" spans="1:7" ht="48.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
@@ -2658,13 +2684,13 @@
       <c r="C45" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D45" s="31">
+      <c r="D45" s="41">
         <f>SUM(C44:C44)</f>
         <v>140</v>
       </c>
-      <c r="E45" s="31"/>
-      <c r="F45" s="31"/>
-      <c r="G45" s="32"/>
+      <c r="E45" s="41"/>
+      <c r="F45" s="41"/>
+      <c r="G45" s="42"/>
     </row>
     <row r="46" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
@@ -2792,13 +2818,13 @@
       <c r="C52" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D52" s="31">
+      <c r="D52" s="41">
         <f>SUM(C46:C51)</f>
         <v>190</v>
       </c>
-      <c r="E52" s="31"/>
-      <c r="F52" s="31"/>
-      <c r="G52" s="32"/>
+      <c r="E52" s="41"/>
+      <c r="F52" s="41"/>
+      <c r="G52" s="42"/>
     </row>
     <row r="53" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
@@ -2873,13 +2899,13 @@
       <c r="C56" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D56" s="31">
+      <c r="D56" s="41">
         <f>SUM(C53:C55)</f>
         <v>140</v>
       </c>
-      <c r="E56" s="31"/>
-      <c r="F56" s="31"/>
-      <c r="G56" s="32"/>
+      <c r="E56" s="41"/>
+      <c r="F56" s="41"/>
+      <c r="G56" s="42"/>
     </row>
     <row r="57" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
@@ -2935,13 +2961,13 @@
       <c r="C59" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D59" s="31">
+      <c r="D59" s="41">
         <f>SUM(C57:C58)</f>
         <v>140</v>
       </c>
-      <c r="E59" s="31"/>
-      <c r="F59" s="31"/>
-      <c r="G59" s="32"/>
+      <c r="E59" s="41"/>
+      <c r="F59" s="41"/>
+      <c r="G59" s="42"/>
     </row>
     <row r="60" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
@@ -3035,13 +3061,13 @@
       <c r="C64" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D64" s="31">
+      <c r="D64" s="41">
         <f>SUM(C60:C63)</f>
         <v>180</v>
       </c>
-      <c r="E64" s="31"/>
-      <c r="F64" s="31"/>
-      <c r="G64" s="32"/>
+      <c r="E64" s="41"/>
+      <c r="F64" s="41"/>
+      <c r="G64" s="42"/>
     </row>
     <row r="65" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
@@ -3152,13 +3178,13 @@
       <c r="C70" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D70" s="31">
+      <c r="D70" s="41">
         <f>SUM(C65:C69)</f>
         <v>145</v>
       </c>
-      <c r="E70" s="31"/>
-      <c r="F70" s="31"/>
-      <c r="G70" s="32"/>
+      <c r="E70" s="41"/>
+      <c r="F70" s="41"/>
+      <c r="G70" s="42"/>
     </row>
     <row r="71" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="s">
@@ -3250,13 +3276,13 @@
       <c r="C75" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D75" s="31">
+      <c r="D75" s="41">
         <f>SUM(C71:C74)</f>
         <v>195</v>
       </c>
-      <c r="E75" s="31"/>
-      <c r="F75" s="31"/>
-      <c r="G75" s="32"/>
+      <c r="E75" s="41"/>
+      <c r="F75" s="41"/>
+      <c r="G75" s="42"/>
     </row>
     <row r="76" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
@@ -3422,7 +3448,7 @@
       <c r="A84" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B84" s="30"/>
+      <c r="B84" s="32"/>
       <c r="C84" s="7">
         <v>5</v>
       </c>
@@ -3447,13 +3473,13 @@
       <c r="C85" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D85" s="31">
+      <c r="D85" s="41">
         <f>SUM(C76:C84)</f>
         <v>215</v>
       </c>
-      <c r="E85" s="31"/>
-      <c r="F85" s="31"/>
-      <c r="G85" s="32"/>
+      <c r="E85" s="41"/>
+      <c r="F85" s="41"/>
+      <c r="G85" s="42"/>
     </row>
     <row r="86" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
@@ -3547,257 +3573,230 @@
       <c r="C90" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D90" s="31">
+      <c r="D90" s="41">
         <f>SUM(C86:C89)</f>
         <v>190</v>
       </c>
-      <c r="E90" s="31"/>
-      <c r="F90" s="31"/>
-      <c r="G90" s="32"/>
-    </row>
-    <row r="91" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="4"/>
-      <c r="B91" s="28"/>
-      <c r="C91" s="5"/>
-      <c r="D91" s="8"/>
-      <c r="E91" s="8"/>
-      <c r="F91" s="22"/>
-      <c r="G91" s="19"/>
-    </row>
-    <row r="92" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="6"/>
+      <c r="E90" s="41"/>
+      <c r="F90" s="41"/>
+      <c r="G90" s="42"/>
+    </row>
+    <row r="91" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B91" s="28">
+        <v>46084</v>
+      </c>
+      <c r="C91" s="5">
+        <v>105</v>
+      </c>
+      <c r="D91" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="E91" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F91" s="23">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="G91" s="8" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="B92" s="29"/>
-      <c r="C92" s="7"/>
-      <c r="D92" s="8"/>
-      <c r="E92" s="8"/>
-      <c r="F92" s="22"/>
-      <c r="G92" s="19"/>
-    </row>
-    <row r="93" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="6"/>
-      <c r="B93" s="29"/>
-      <c r="C93" s="7"/>
-      <c r="D93" s="8"/>
-      <c r="E93" s="8"/>
-      <c r="F93" s="7"/>
-      <c r="G93" s="19"/>
+      <c r="C92" s="7">
+        <v>85</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="E92" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F92" s="23">
+        <v>0.47569444444444442</v>
+      </c>
+      <c r="G92" s="8" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B93" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="C93" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="D93" s="41">
+        <f>SUM(C91:C92)</f>
+        <v>190</v>
+      </c>
+      <c r="E93" s="41"/>
+      <c r="F93" s="41"/>
+      <c r="G93" s="42"/>
     </row>
     <row r="94" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="6"/>
-      <c r="B94" s="29"/>
-      <c r="C94" s="7"/>
+      <c r="A94" s="4"/>
+      <c r="B94" s="28"/>
+      <c r="C94" s="5"/>
       <c r="D94" s="8"/>
       <c r="E94" s="8"/>
-      <c r="F94" s="7"/>
+      <c r="F94" s="22"/>
       <c r="G94" s="19"/>
     </row>
-    <row r="95" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A95" s="9"/>
-      <c r="B95" s="30"/>
-      <c r="C95" s="9"/>
+    <row r="95" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="6"/>
+      <c r="B95" s="29"/>
+      <c r="C95" s="7"/>
       <c r="D95" s="8"/>
-      <c r="E95" s="10"/>
-      <c r="F95" s="7"/>
+      <c r="E95" s="8"/>
+      <c r="F95" s="22"/>
       <c r="G95" s="19"/>
     </row>
-    <row r="96" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="B96" s="17" t="s">
-        <v>141</v>
-      </c>
-      <c r="C96" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="D96" s="31">
-        <f>SUM(C91:C95)</f>
-        <v>0</v>
-      </c>
-      <c r="E96" s="31"/>
-      <c r="F96" s="31"/>
-      <c r="G96" s="32"/>
+    <row r="96" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="6"/>
+      <c r="B96" s="29"/>
+      <c r="C96" s="7"/>
+      <c r="D96" s="8"/>
+      <c r="E96" s="8"/>
+      <c r="F96" s="7"/>
+      <c r="G96" s="19"/>
     </row>
     <row r="97" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="4"/>
-      <c r="B97" s="28"/>
-      <c r="C97" s="5"/>
+      <c r="A97" s="6"/>
+      <c r="B97" s="29"/>
+      <c r="C97" s="7"/>
       <c r="D97" s="8"/>
       <c r="E97" s="8"/>
-      <c r="F97" s="22"/>
+      <c r="F97" s="7"/>
       <c r="G97" s="19"/>
     </row>
-    <row r="98" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="6"/>
-      <c r="B98" s="29"/>
-      <c r="C98" s="7"/>
+    <row r="98" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="9"/>
+      <c r="B98" s="32"/>
+      <c r="C98" s="9"/>
       <c r="D98" s="8"/>
-      <c r="E98" s="8"/>
-      <c r="F98" s="22"/>
+      <c r="E98" s="10"/>
+      <c r="F98" s="7"/>
       <c r="G98" s="19"/>
     </row>
-    <row r="99" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="6"/>
-      <c r="B99" s="29"/>
-      <c r="C99" s="7"/>
-      <c r="D99" s="8"/>
-      <c r="E99" s="8"/>
-      <c r="F99" s="7"/>
-      <c r="G99" s="19"/>
+    <row r="99" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B99" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="C99" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="D99" s="41">
+        <f>SUM(C94:C98)</f>
+        <v>0</v>
+      </c>
+      <c r="E99" s="41"/>
+      <c r="F99" s="41"/>
+      <c r="G99" s="42"/>
     </row>
     <row r="100" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="6"/>
-      <c r="B100" s="29"/>
-      <c r="C100" s="7"/>
+      <c r="A100" s="4"/>
+      <c r="B100" s="28"/>
+      <c r="C100" s="5"/>
       <c r="D100" s="8"/>
       <c r="E100" s="8"/>
-      <c r="F100" s="7"/>
+      <c r="F100" s="22"/>
       <c r="G100" s="19"/>
     </row>
-    <row r="101" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="9"/>
-      <c r="B101" s="30"/>
-      <c r="C101" s="9"/>
+    <row r="101" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="6"/>
+      <c r="B101" s="29"/>
+      <c r="C101" s="7"/>
       <c r="D101" s="8"/>
-      <c r="E101" s="10"/>
-      <c r="F101" s="7"/>
+      <c r="E101" s="8"/>
+      <c r="F101" s="22"/>
       <c r="G101" s="19"/>
     </row>
-    <row r="102" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="B102" s="17" t="s">
-        <v>148</v>
-      </c>
-      <c r="C102" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="D102" s="31">
-        <f>SUM(C97:C101)</f>
-        <v>0</v>
-      </c>
-      <c r="E102" s="31"/>
-      <c r="F102" s="31"/>
-      <c r="G102" s="32"/>
+    <row r="102" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="6"/>
+      <c r="B102" s="29"/>
+      <c r="C102" s="7"/>
+      <c r="D102" s="8"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="7"/>
+      <c r="G102" s="19"/>
     </row>
     <row r="103" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="4"/>
-      <c r="B103" s="28"/>
-      <c r="C103" s="5"/>
+      <c r="A103" s="6"/>
+      <c r="B103" s="29"/>
+      <c r="C103" s="7"/>
       <c r="D103" s="8"/>
       <c r="E103" s="8"/>
-      <c r="F103" s="22"/>
+      <c r="F103" s="7"/>
       <c r="G103" s="19"/>
     </row>
-    <row r="104" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="6"/>
-      <c r="B104" s="29"/>
-      <c r="C104" s="7"/>
+    <row r="104" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="9"/>
+      <c r="B104" s="32"/>
+      <c r="C104" s="9"/>
       <c r="D104" s="8"/>
-      <c r="E104" s="8"/>
-      <c r="F104" s="22"/>
+      <c r="E104" s="10"/>
+      <c r="F104" s="7"/>
       <c r="G104" s="19"/>
     </row>
-    <row r="105" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="6"/>
-      <c r="B105" s="29"/>
-      <c r="C105" s="7"/>
-      <c r="D105" s="8"/>
-      <c r="E105" s="8"/>
-      <c r="F105" s="7"/>
-      <c r="G105" s="19"/>
-    </row>
-    <row r="106" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A106" s="6"/>
-      <c r="B106" s="29"/>
-      <c r="C106" s="7"/>
-      <c r="D106" s="8"/>
-      <c r="E106" s="8"/>
-      <c r="F106" s="7"/>
-      <c r="G106" s="19"/>
-    </row>
-    <row r="107" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A107" s="9"/>
-      <c r="B107" s="30"/>
-      <c r="C107" s="9"/>
-      <c r="D107" s="8"/>
-      <c r="E107" s="10"/>
-      <c r="F107" s="7"/>
-      <c r="G107" s="19"/>
-    </row>
-    <row r="108" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A108" s="11" t="s">
+    <row r="105" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A105" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="B108" s="17" t="s">
+      <c r="B105" s="17" t="s">
         <v>149</v>
       </c>
-      <c r="C108" s="17" t="s">
+      <c r="C105" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D108" s="31">
-        <f>SUM(C103:C107)</f>
+      <c r="D105" s="41">
+        <f>SUM(C100:C104)</f>
         <v>0</v>
       </c>
-      <c r="E108" s="31"/>
-      <c r="F108" s="31"/>
-      <c r="G108" s="32"/>
-    </row>
-    <row r="109" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A109" s="42" t="s">
+      <c r="E105" s="41"/>
+      <c r="F105" s="41"/>
+      <c r="G105" s="42"/>
+    </row>
+    <row r="106" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A106" s="30" t="s">
         <v>111</v>
       </c>
-      <c r="B109" s="43"/>
-      <c r="C109" s="12">
-        <f>MROUND(SUM(C6:C108) /60,0.2)</f>
-        <v>45.2</v>
-      </c>
-      <c r="D109" s="13"/>
-      <c r="E109" s="18"/>
-      <c r="F109" s="20"/>
-      <c r="G109" s="14"/>
-    </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A110" s="15"/>
-    </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A111" s="15"/>
+      <c r="B106" s="31"/>
+      <c r="C106" s="12">
+        <f>MROUND(SUM(C6:C105) /60,0.2)</f>
+        <v>48.400000000000006</v>
+      </c>
+      <c r="D106" s="13"/>
+      <c r="E106" s="18"/>
+      <c r="F106" s="20"/>
+      <c r="G106" s="14"/>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A107" s="15"/>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A108" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="B23:B25"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="A109:B109"/>
-    <mergeCell ref="B31:B39"/>
-    <mergeCell ref="B103:B107"/>
-    <mergeCell ref="B46:B51"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="B71:B74"/>
-    <mergeCell ref="B65:B69"/>
-    <mergeCell ref="B53:B55"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="B60:B63"/>
-    <mergeCell ref="B86:B89"/>
-    <mergeCell ref="B97:B101"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="D9:G9"/>
-    <mergeCell ref="D15:G15"/>
-    <mergeCell ref="D19:G19"/>
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="B6:B8"/>
-    <mergeCell ref="B10:B14"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="D108:G108"/>
+    <mergeCell ref="D22:G22"/>
+    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="D30:G30"/>
+    <mergeCell ref="D40:G40"/>
+    <mergeCell ref="B76:B84"/>
+    <mergeCell ref="D105:G105"/>
     <mergeCell ref="D52:G52"/>
     <mergeCell ref="D43:G43"/>
     <mergeCell ref="D45:G45"/>
@@ -3808,21 +3807,47 @@
     <mergeCell ref="D64:G64"/>
     <mergeCell ref="D85:G85"/>
     <mergeCell ref="D90:G90"/>
-    <mergeCell ref="D102:G102"/>
-    <mergeCell ref="B91:B95"/>
-    <mergeCell ref="D96:G96"/>
-    <mergeCell ref="D22:G22"/>
-    <mergeCell ref="D26:G26"/>
-    <mergeCell ref="D30:G30"/>
-    <mergeCell ref="D40:G40"/>
-    <mergeCell ref="B76:B84"/>
+    <mergeCell ref="D99:G99"/>
+    <mergeCell ref="D93:G93"/>
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="D15:G15"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="B10:B14"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="B23:B25"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="A106:B106"/>
+    <mergeCell ref="B31:B39"/>
+    <mergeCell ref="B100:B104"/>
+    <mergeCell ref="B46:B51"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="B71:B74"/>
+    <mergeCell ref="B65:B69"/>
+    <mergeCell ref="B53:B55"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="B60:B63"/>
+    <mergeCell ref="B86:B89"/>
+    <mergeCell ref="B94:B98"/>
+    <mergeCell ref="B91:B92"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C103:C107 C27:C29 C23:C25 C16:C18 B6 C10:C14 C20:C21 C6:C8 C31:C39 C41:C42 C44 C46:C51 C71:C74 C53:C55 C60:C63 C57:C58 C65:C69 C76:C84 C86:C89 C97:C101 C91:C95" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C100:C104 C27:C29 C23:C25 C16:C18 B6 C10:C14 C20:C21 C6:C8 C31:C39 C41:C42 C44 C46:C51 C71:C74 C53:C55 C60:C63 C57:C58 C65:C69 C76:C84 C86:C89 C94:C98 C91:C92" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B10:B14 B16:B18 B20:B21 B103:B107 B27:B29 B23:B25 B31:B39 B41:B42 B44 B46:B51 B71:B74 B53:B55 B60:B63 B57:B58 B65:B69 B76 B86:B89 B97:B101 B91:B95" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B10:B14 B16:B18 B20:B21 B100:B104 B27:B29 B23:B25 B31:B39 B41:B42 B44 B46:B51 B71:B74 B53:B55 B60:B63 B57:B58 B65:B69 B76 B86:B89 B94:B98 B91:B92" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -3842,7 +3867,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="109" operator="equal" id="{6BC2577B-BDA3-4B48-8F95-0F2177F9264F}">
+          <x14:cfRule type="cellIs" priority="111" operator="equal" id="{6BC2577B-BDA3-4B48-8F95-0F2177F9264F}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3852,10 +3877,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>A4:E8 A10:E14 A16:E18 A20:E21 A23:E25 A27:E29 A31:E39 A103:E107 A109:E1048576 A44:E44 A41:E42 A46:E51 A71:E74 A65:E69 A60:E63 A57:E58 A53:E55 A86:E89 A76:E76 C77:E84 A97:E101 A91:E95 A1:D2 F1:F3 A3 D3 G4:G5 G7:G8 A9:D9 A15:D15 A19:D19 A22:D22 A26:D26 A30:D30 A40:D40 A43:D43 A45:D45 A52:D52 A56:D56 A59:D59 A64:D64 A70:D70 A75:D75 A77:A84 A85:D85 A90:D90 A96:D96 A102:D102 A108:D108 G109:G1048576</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="108" operator="equal" id="{9C6C644F-7238-453A-BC69-B42FAB3A2FA5}">
+          <xm:sqref>A4:E8 A10:E14 A16:E18 A20:E21 A23:E25 A27:E29 A31:E39 A100:E104 A106:E1048576 A44:E44 A41:E42 A46:E51 A71:E74 A65:E69 A60:E63 A57:E58 A53:E55 A86:E89 A76:E76 C77:E84 A94:E98 A91:E92 A1:D2 F1:F3 A3 D3 G4:G5 G7:G8 A9:D9 A15:D15 A19:D19 A22:D22 A26:D26 A30:D30 A40:D40 A43:D43 A45:D45 A52:D52 A56:D56 A59:D59 A64:D64 A70:D70 A75:D75 A77:A84 A85:D85 A90:D90 A93:D93 A99:D99 A105:D105 G106:G1048576</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="110" operator="equal" id="{9C6C644F-7238-453A-BC69-B42FAB3A2FA5}">
             <xm:f>Restrictions!$A$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3865,7 +3890,17 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="111" operator="equal" id="{29EA468D-F98D-4D41-AA55-B63DA0941363}">
+          <x14:cfRule type="cellIs" priority="112" operator="equal" id="{6DE85145-1CAE-407F-B647-4C9B303613C7}">
+            <xm:f>Restrictions!$C$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="113" operator="equal" id="{29EA468D-F98D-4D41-AA55-B63DA0941363}">
             <xm:f>Restrictions!$D$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3875,7 +3910,20 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="110" operator="equal" id="{6DE85145-1CAE-407F-B647-4C9B303613C7}">
+          <xm:sqref>E4:E8 E10:E14 E16:E18 E20:E21 E23:E25 E27:E29 E31:E39 E100:E104 E106:E1048576</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="79" operator="equal" id="{84E995EC-6FB3-447D-B7B4-F39F6B4AAF45}">
+            <xm:f>Restrictions!$A$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B050"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="80" operator="equal" id="{B6903E1B-29F5-497F-B030-3589B8B337A1}">
             <xm:f>Restrictions!$C$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3885,10 +3933,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E4:E8 E10:E14 E16:E18 E20:E21 E23:E25 E27:E29 E31:E39 E103:E107 E109:E1048576</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="79" operator="equal" id="{DA16BC0E-098E-492D-9DD4-7AE32F5A0B66}">
+          <x14:cfRule type="cellIs" priority="81" operator="equal" id="{DA16BC0E-098E-492D-9DD4-7AE32F5A0B66}">
             <xm:f>Restrictions!$D$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3898,7 +3943,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="77" operator="equal" id="{84E995EC-6FB3-447D-B7B4-F39F6B4AAF45}">
+          <xm:sqref>E41:E42</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="83" operator="equal" id="{2763426F-5E05-4AE5-BAB9-6155B44E42F3}">
             <xm:f>Restrictions!$A$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3908,7 +3956,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="78" operator="equal" id="{B6903E1B-29F5-497F-B030-3589B8B337A1}">
+          <x14:cfRule type="cellIs" priority="84" operator="equal" id="{29283CD5-B4A3-4A92-85FA-0825B9BB0F20}">
             <xm:f>Restrictions!$C$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3918,10 +3966,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E41:E42</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="83" operator="equal" id="{FFFCA022-7518-426F-AC53-14AA2D86A5EB}">
+          <x14:cfRule type="cellIs" priority="85" operator="equal" id="{FFFCA022-7518-426F-AC53-14AA2D86A5EB}">
             <xm:f>Restrictions!$D$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3931,7 +3976,20 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="82" operator="equal" id="{29283CD5-B4A3-4A92-85FA-0825B9BB0F20}">
+          <xm:sqref>E44</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="71" operator="equal" id="{55BA1703-E0F0-4534-AC5F-5524C52012B8}">
+            <xm:f>Restrictions!$A$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B050"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="72" operator="equal" id="{8AA9BDE2-93E5-4C8F-8ABB-C8A37EF6C1F7}">
             <xm:f>Restrictions!$C$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3941,7 +3999,20 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="81" operator="equal" id="{2763426F-5E05-4AE5-BAB9-6155B44E42F3}">
+          <x14:cfRule type="cellIs" priority="73" operator="equal" id="{7CBCFDCF-397F-4B71-B6B1-D6B8B3D995CF}">
+            <xm:f>Restrictions!$D$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>E46:E51</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="51" operator="equal" id="{38CC099F-2CFB-4F51-BCC6-9A8C062F12D6}">
             <xm:f>Restrictions!$A$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3951,10 +4022,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E44</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="70" operator="equal" id="{8AA9BDE2-93E5-4C8F-8ABB-C8A37EF6C1F7}">
+          <x14:cfRule type="cellIs" priority="52" operator="equal" id="{97B7369B-F3E2-421C-8B11-B917735F9E01}">
             <xm:f>Restrictions!$C$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3964,7 +4032,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="71" operator="equal" id="{7CBCFDCF-397F-4B71-B6B1-D6B8B3D995CF}">
+          <x14:cfRule type="cellIs" priority="53" operator="equal" id="{9BE9A0C0-12EE-4A06-AA91-2B2C7773C591}">
             <xm:f>Restrictions!$D$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3974,7 +4042,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="69" operator="equal" id="{55BA1703-E0F0-4534-AC5F-5524C52012B8}">
+          <xm:sqref>E53:E55</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="55" operator="equal" id="{CE91AE07-0A4B-4CA1-864E-4494D1FD3F2D}">
             <xm:f>Restrictions!$A$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3984,10 +4055,17 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E46:E51</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="51" operator="equal" id="{9BE9A0C0-12EE-4A06-AA91-2B2C7773C591}">
+          <x14:cfRule type="cellIs" priority="56" operator="equal" id="{E33B63BE-9C2D-46FB-840B-160E77C144D1}">
+            <xm:f>Restrictions!$C$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="57" operator="equal" id="{06F1F730-9D3E-44F6-9858-23332EAE481C}">
             <xm:f>Restrictions!$D$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3997,7 +4075,20 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="50" operator="equal" id="{97B7369B-F3E2-421C-8B11-B917735F9E01}">
+          <xm:sqref>E57:E58</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="59" operator="equal" id="{6138D6EC-9477-4522-A720-100D44F804C5}">
+            <xm:f>Restrictions!$A$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B050"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="60" operator="equal" id="{7FB697E4-A1F6-44CC-8422-CFE46191EC29}">
             <xm:f>Restrictions!$C$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4007,7 +4098,20 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="49" operator="equal" id="{38CC099F-2CFB-4F51-BCC6-9A8C062F12D6}">
+          <x14:cfRule type="cellIs" priority="61" operator="equal" id="{F3D48842-32E0-470D-8962-C942EB8B670B}">
+            <xm:f>Restrictions!$D$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>E60:E63</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="63" operator="equal" id="{CF4E2A7B-2831-4A8E-8CB0-05A3819B6512}">
             <xm:f>Restrictions!$A$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4017,10 +4121,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E53:E55</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="54" operator="equal" id="{E33B63BE-9C2D-46FB-840B-160E77C144D1}">
+          <x14:cfRule type="cellIs" priority="64" operator="equal" id="{5A6DBF38-AB31-41CF-92EB-6F71330B8A51}">
             <xm:f>Restrictions!$C$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4030,7 +4131,20 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="53" operator="equal" id="{CE91AE07-0A4B-4CA1-864E-4494D1FD3F2D}">
+          <x14:cfRule type="cellIs" priority="65" operator="equal" id="{806E81D0-33D7-43D5-9F66-9ACF5303AA2B}">
+            <xm:f>Restrictions!$D$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>E65:E69</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="67" operator="equal" id="{EC003FB1-6A08-40D6-88B1-588BCE936C35}">
             <xm:f>Restrictions!$A$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4040,7 +4154,17 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="55" operator="equal" id="{06F1F730-9D3E-44F6-9858-23332EAE481C}">
+          <x14:cfRule type="cellIs" priority="68" operator="equal" id="{CCF6CA8D-69A5-48BE-8938-2E3B52B06A90}">
+            <xm:f>Restrictions!$C$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="69" operator="equal" id="{5E85ED66-7E81-44BB-AFFF-3FBE898F7448}">
             <xm:f>Restrictions!$D$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4050,10 +4174,30 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E57:E58</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="59" operator="equal" id="{F3D48842-32E0-470D-8962-C942EB8B670B}">
+          <xm:sqref>E71:E74</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="20" operator="equal" id="{42B27148-AE7C-4BA1-B993-B3037B69F92A}">
+            <xm:f>Restrictions!$A$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B050"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="21" operator="equal" id="{CAD63670-76D8-46C3-9428-FF1328E16D90}">
+            <xm:f>Restrictions!$C$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="22" operator="equal" id="{5EE1483C-C8AF-4BC8-96C2-1FBDBB50C066}">
             <xm:f>Restrictions!$D$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4063,7 +4207,20 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="58" operator="equal" id="{7FB697E4-A1F6-44CC-8422-CFE46191EC29}">
+          <xm:sqref>E76:E84</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="25" operator="equal" id="{8A959092-8A6B-4A91-99D1-8110E43AA729}">
+            <xm:f>Restrictions!$A$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B050"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="26" operator="equal" id="{F801D24C-AFDA-4757-9BC6-FB24B4DE466D}">
             <xm:f>Restrictions!$C$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4073,7 +4230,20 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="57" operator="equal" id="{6138D6EC-9477-4522-A720-100D44F804C5}">
+          <x14:cfRule type="cellIs" priority="27" operator="equal" id="{8CF84F96-ED65-491E-B676-DA2F761CE9EB}">
+            <xm:f>Restrictions!$D$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>E86:E89</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{92E62023-F404-4026-AD69-5B76EB0BDAE8}">
             <xm:f>Restrictions!$A$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4083,10 +4253,30 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E60:E63</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="61" operator="equal" id="{CF4E2A7B-2831-4A8E-8CB0-05A3819B6512}">
+          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{9E114EAB-BD08-4433-A88A-51FDBB871F00}">
+            <xm:f>Restrictions!$C$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{5CAB61E4-56FF-4285-A4C9-A33737017E3A}">
+            <xm:f>Restrictions!$D$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>E91:E92</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{A66F7540-0CD1-4EF9-B347-2CABE04E932F}">
             <xm:f>Restrictions!$A$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4096,7 +4286,17 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="63" operator="equal" id="{806E81D0-33D7-43D5-9F66-9ACF5303AA2B}">
+          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{E10A4C2F-1FA6-426F-A318-4C7EFBFBAD06}">
+            <xm:f>Restrictions!$C$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="10" operator="equal" id="{59C9B578-9F2D-494D-BED9-807E89EADAB8}">
             <xm:f>Restrictions!$D$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4106,185 +4306,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="62" operator="equal" id="{5A6DBF38-AB31-41CF-92EB-6F71330B8A51}">
-            <xm:f>Restrictions!$C$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFC000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>E65:E69</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="66" operator="equal" id="{CCF6CA8D-69A5-48BE-8938-2E3B52B06A90}">
-            <xm:f>Restrictions!$C$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFC000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="67" operator="equal" id="{5E85ED66-7E81-44BB-AFFF-3FBE898F7448}">
-            <xm:f>Restrictions!$D$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFF0000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="65" operator="equal" id="{EC003FB1-6A08-40D6-88B1-588BCE936C35}">
-            <xm:f>Restrictions!$A$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B050"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>E71:E74</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="20" operator="equal" id="{5EE1483C-C8AF-4BC8-96C2-1FBDBB50C066}">
-            <xm:f>Restrictions!$D$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFF0000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="19" operator="equal" id="{CAD63670-76D8-46C3-9428-FF1328E16D90}">
-            <xm:f>Restrictions!$C$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFC000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="18" operator="equal" id="{42B27148-AE7C-4BA1-B993-B3037B69F92A}">
-            <xm:f>Restrictions!$A$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B050"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>E76:E84</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="24" operator="equal" id="{F801D24C-AFDA-4757-9BC6-FB24B4DE466D}">
-            <xm:f>Restrictions!$C$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFC000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="23" operator="equal" id="{8A959092-8A6B-4A91-99D1-8110E43AA729}">
-            <xm:f>Restrictions!$A$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B050"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="25" operator="equal" id="{8CF84F96-ED65-491E-B676-DA2F761CE9EB}">
-            <xm:f>Restrictions!$D$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFF0000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>E86:E89</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{92E62023-F404-4026-AD69-5B76EB0BDAE8}">
-            <xm:f>Restrictions!$A$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B050"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{9E114EAB-BD08-4433-A88A-51FDBB871F00}">
-            <xm:f>Restrictions!$C$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFC000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{5CAB61E4-56FF-4285-A4C9-A33737017E3A}">
-            <xm:f>Restrictions!$D$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFF0000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>E91:E95</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{A66F7540-0CD1-4EF9-B347-2CABE04E932F}">
-            <xm:f>Restrictions!$A$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B050"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{59C9B578-9F2D-494D-BED9-807E89EADAB8}">
-            <xm:f>Restrictions!$D$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFF0000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{E10A4C2F-1FA6-426F-A318-4C7EFBFBAD06}">
-            <xm:f>Restrictions!$C$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFC000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>E97:E101</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="105" operator="containsText" id="{FD0F452B-B2F8-4F75-A8CD-A69AC0834E64}">
+          <xm:sqref>E94:E98</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="107" operator="containsText" id="{FD0F452B-B2F8-4F75-A8CD-A69AC0834E64}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F6)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4298,7 +4323,7 @@
           <xm:sqref>F6:F8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="103" operator="containsText" id="{6407061A-B268-44CE-A52C-133739941B16}">
+          <x14:cfRule type="containsText" priority="105" operator="containsText" id="{6407061A-B268-44CE-A52C-133739941B16}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F16)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4312,7 +4337,7 @@
           <xm:sqref>F16:F18</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="102" operator="containsText" id="{756A584A-6AAC-4559-9F27-A59B4EFD7F34}">
+          <x14:cfRule type="containsText" priority="104" operator="containsText" id="{756A584A-6AAC-4559-9F27-A59B4EFD7F34}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F20)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4326,7 +4351,7 @@
           <xm:sqref>F20:F21</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="101" operator="containsText" id="{E988FD75-2909-4816-91C7-1018002A435D}">
+          <x14:cfRule type="containsText" priority="103" operator="containsText" id="{E988FD75-2909-4816-91C7-1018002A435D}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F23)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4340,7 +4365,7 @@
           <xm:sqref>F23 F24:G24 F25</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="100" operator="containsText" id="{D5B6D5DF-9E2A-4C4B-BA82-97D983766AEE}">
+          <x14:cfRule type="containsText" priority="102" operator="containsText" id="{D5B6D5DF-9E2A-4C4B-BA82-97D983766AEE}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F27)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4354,7 +4379,7 @@
           <xm:sqref>F27:F28 F29:G29</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="80" operator="containsText" id="{58D84678-3AF3-4F30-A017-BCF30ADC23B9}">
+          <x14:cfRule type="containsText" priority="82" operator="containsText" id="{58D84678-3AF3-4F30-A017-BCF30ADC23B9}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F44)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4368,7 +4393,7 @@
           <xm:sqref>F44</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="48" operator="containsText" id="{2CEED9A6-BF96-4A7D-A6A3-A1CBCB1BBB33}">
+          <x14:cfRule type="containsText" priority="50" operator="containsText" id="{2CEED9A6-BF96-4A7D-A6A3-A1CBCB1BBB33}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F53)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4382,7 +4407,7 @@
           <xm:sqref>F53 F54:G54 F55</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="52" operator="containsText" id="{9846E030-D336-4ABF-8549-0B217B1EE9C0}">
+          <x14:cfRule type="containsText" priority="54" operator="containsText" id="{9846E030-D336-4ABF-8549-0B217B1EE9C0}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F57)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4396,7 +4421,7 @@
           <xm:sqref>F57:F58</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="56" operator="containsText" id="{C331D7E9-51D1-4558-86A6-2DDD97E5F51B}">
+          <x14:cfRule type="containsText" priority="58" operator="containsText" id="{C331D7E9-51D1-4558-86A6-2DDD97E5F51B}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F60)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4410,7 +4435,7 @@
           <xm:sqref>F60 F61:G62 F63</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="64" operator="containsText" id="{A87BC3C4-539A-4D6D-94C0-DF4DFEA06C8A}">
+          <x14:cfRule type="containsText" priority="66" operator="containsText" id="{A87BC3C4-539A-4D6D-94C0-DF4DFEA06C8A}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F71)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4424,7 +4449,7 @@
           <xm:sqref>F71 F72:G74</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="21" operator="containsText" id="{94391AE6-F1AE-42D1-AF78-4812D68E41C4}">
+          <x14:cfRule type="containsText" priority="23" operator="containsText" id="{94391AE6-F1AE-42D1-AF78-4812D68E41C4}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F84)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4438,7 +4463,7 @@
           <xm:sqref>F84</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="104" operator="containsText" id="{88417B48-EA26-4D48-9EFE-B6A1E5C426AE}">
+          <x14:cfRule type="containsText" priority="106" operator="containsText" id="{88417B48-EA26-4D48-9EFE-B6A1E5C426AE}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F10)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4452,7 +4477,7 @@
           <xm:sqref>F10:G10 F11:F12 F13:G13 F14</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="99" operator="containsText" id="{1555D56B-E8B5-4F0A-9D80-B2C1016EB105}">
+          <x14:cfRule type="containsText" priority="101" operator="containsText" id="{1555D56B-E8B5-4F0A-9D80-B2C1016EB105}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F31)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4466,7 +4491,7 @@
           <xm:sqref>F31:G31 F32</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="88" operator="containsText" id="{F174B00B-9E6F-49FA-9EE7-95FA16CF0425}">
+          <x14:cfRule type="containsText" priority="90" operator="containsText" id="{F174B00B-9E6F-49FA-9EE7-95FA16CF0425}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F33)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4480,7 +4505,7 @@
           <xm:sqref>F33:G38 F39</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="76" operator="containsText" id="{4AF076A7-8EED-499A-B340-9301C9A23B63}">
+          <x14:cfRule type="containsText" priority="78" operator="containsText" id="{4AF076A7-8EED-499A-B340-9301C9A23B63}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F41)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4494,7 +4519,7 @@
           <xm:sqref>F41:G41 F42</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="68" operator="containsText" id="{1E89304F-1BDF-40FA-83E9-2770D86CCD7D}">
+          <x14:cfRule type="containsText" priority="70" operator="containsText" id="{1E89304F-1BDF-40FA-83E9-2770D86CCD7D}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F46)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4508,7 +4533,7 @@
           <xm:sqref>F46:G51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="60" operator="containsText" id="{FBCB4E68-F50D-4BE4-8CEE-A9CE7EAE06EE}">
+          <x14:cfRule type="containsText" priority="62" operator="containsText" id="{FBCB4E68-F50D-4BE4-8CEE-A9CE7EAE06EE}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F65)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4522,7 +4547,7 @@
           <xm:sqref>F65:G69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="34" operator="containsText" id="{3688DB4D-873A-4169-BE4C-08434A027D62}">
+          <x14:cfRule type="containsText" priority="36" operator="containsText" id="{3688DB4D-873A-4169-BE4C-08434A027D62}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F76)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4536,7 +4561,7 @@
           <xm:sqref>F76:G76 F77 F78:G79 F80</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="27" operator="containsText" id="{1CA0FC1F-6CFD-462C-912C-B25E380596FE}">
+          <x14:cfRule type="containsText" priority="29" operator="containsText" id="{1CA0FC1F-6CFD-462C-912C-B25E380596FE}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F81)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4550,7 +4575,7 @@
           <xm:sqref>F81:G83</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="14" operator="containsText" id="{6EAE5B84-F778-418F-A1B7-BC9BA100112D}">
+          <x14:cfRule type="containsText" priority="16" operator="containsText" id="{6EAE5B84-F778-418F-A1B7-BC9BA100112D}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F86)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4564,7 +4589,7 @@
           <xm:sqref>F86:G89</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" operator="containsText" id="{49774D53-9CD8-4DDA-86D7-61DDC39694A2}">
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{49774D53-9CD8-4DDA-86D7-61DDC39694A2}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F91)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4575,11 +4600,11 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>F91:G95</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="5" operator="containsText" id="{EC18E800-531E-417C-9061-1973EA038CA3}">
-            <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F97)))</xm:f>
+          <xm:sqref>F91:F92</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="7" operator="containsText" id="{EC18E800-531E-417C-9061-1973EA038CA3}">
+            <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F94)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4589,11 +4614,11 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>F97:G101</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="98" operator="containsText" id="{2F0F41F7-8C93-48A6-B013-C45F8E29AE34}">
-            <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F103)))</xm:f>
+          <xm:sqref>F94:G98</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="100" operator="containsText" id="{2F0F41F7-8C93-48A6-B013-C45F8E29AE34}">
+            <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F100)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4603,10 +4628,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>F103:G107</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="97" operator="equal" id="{C81CB296-EBDE-4E68-996A-22E647E300C9}">
+          <xm:sqref>F100:G104</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="99" operator="equal" id="{C81CB296-EBDE-4E68-996A-22E647E300C9}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4619,7 +4644,7 @@
           <xm:sqref>G11:G12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="96" operator="equal" id="{C6523CE4-984A-4BEA-B850-BBE212DEC1BD}">
+          <x14:cfRule type="cellIs" priority="98" operator="equal" id="{C6523CE4-984A-4BEA-B850-BBE212DEC1BD}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4632,7 +4657,7 @@
           <xm:sqref>G14</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="95" operator="equal" id="{34CA0963-7227-4B81-A491-AF5EBF6948E0}">
+          <x14:cfRule type="cellIs" priority="97" operator="equal" id="{34CA0963-7227-4B81-A491-AF5EBF6948E0}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4645,7 +4670,7 @@
           <xm:sqref>G16:G18</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="94" operator="equal" id="{0137ED0B-0223-4A2D-BBA6-66B7E7B0177B}">
+          <x14:cfRule type="cellIs" priority="96" operator="equal" id="{0137ED0B-0223-4A2D-BBA6-66B7E7B0177B}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4658,7 +4683,7 @@
           <xm:sqref>G20:G21</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="93" operator="equal" id="{0559BE0C-06E8-4BF0-855B-46B347A65A43}">
+          <x14:cfRule type="cellIs" priority="95" operator="equal" id="{0559BE0C-06E8-4BF0-855B-46B347A65A43}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4671,7 +4696,7 @@
           <xm:sqref>G23</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="92" operator="equal" id="{A10A680C-18B8-4576-98EE-F30E41E55578}">
+          <x14:cfRule type="cellIs" priority="94" operator="equal" id="{A10A680C-18B8-4576-98EE-F30E41E55578}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4684,7 +4709,7 @@
           <xm:sqref>G25</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="91" operator="equal" id="{EE200D4C-87A3-41C0-AADC-DBA0F1BBC7B2}">
+          <x14:cfRule type="cellIs" priority="93" operator="equal" id="{EE200D4C-87A3-41C0-AADC-DBA0F1BBC7B2}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4697,7 +4722,7 @@
           <xm:sqref>G27:G28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="90" operator="equal" id="{11814DC1-0D86-496F-AEC1-5E73F0134CB6}">
+          <x14:cfRule type="cellIs" priority="92" operator="equal" id="{11814DC1-0D86-496F-AEC1-5E73F0134CB6}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4710,7 +4735,7 @@
           <xm:sqref>G32</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="75" operator="equal" id="{267A3B51-36A4-44DF-B2E6-F06E71682E5F}">
+          <x14:cfRule type="cellIs" priority="77" operator="equal" id="{267A3B51-36A4-44DF-B2E6-F06E71682E5F}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4723,7 +4748,7 @@
           <xm:sqref>G39</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="74" operator="equal" id="{0FA35E81-D3C4-44FE-9341-C74ABA01B1FF}">
+          <x14:cfRule type="cellIs" priority="76" operator="equal" id="{0FA35E81-D3C4-44FE-9341-C74ABA01B1FF}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4736,7 +4761,7 @@
           <xm:sqref>G42</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="73" operator="equal" id="{E1E75134-FA7A-4AB7-9C7B-BBBAB5BA6AE8}">
+          <x14:cfRule type="cellIs" priority="75" operator="equal" id="{E1E75134-FA7A-4AB7-9C7B-BBBAB5BA6AE8}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4749,7 +4774,7 @@
           <xm:sqref>G44</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="47" operator="equal" id="{7506C776-F73B-475A-A848-0E98C716D28F}">
+          <x14:cfRule type="cellIs" priority="49" operator="equal" id="{7506C776-F73B-475A-A848-0E98C716D28F}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4762,7 +4787,7 @@
           <xm:sqref>G53</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="46" operator="equal" id="{EEDBCFEE-8EE0-4370-A603-3DD0D0A3C004}">
+          <x14:cfRule type="cellIs" priority="48" operator="equal" id="{EEDBCFEE-8EE0-4370-A603-3DD0D0A3C004}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4775,7 +4800,7 @@
           <xm:sqref>G55</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="45" operator="equal" id="{EBD16DC6-D1FA-4FC5-B74B-CA3CF0413675}">
+          <x14:cfRule type="cellIs" priority="47" operator="equal" id="{EBD16DC6-D1FA-4FC5-B74B-CA3CF0413675}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4788,7 +4813,7 @@
           <xm:sqref>G57:G58</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="44" operator="equal" id="{CB5C53FD-3D5D-4030-A78E-D6ACDDA5D5F7}">
+          <x14:cfRule type="cellIs" priority="46" operator="equal" id="{CB5C53FD-3D5D-4030-A78E-D6ACDDA5D5F7}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4801,7 +4826,7 @@
           <xm:sqref>G60</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="43" operator="equal" id="{28414CE1-4551-493E-98F2-E4708C3326DE}">
+          <x14:cfRule type="cellIs" priority="45" operator="equal" id="{28414CE1-4551-493E-98F2-E4708C3326DE}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4814,7 +4839,7 @@
           <xm:sqref>G63</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="42" operator="equal" id="{19A160C2-6897-43F9-AB25-0B60E506490B}">
+          <x14:cfRule type="cellIs" priority="44" operator="equal" id="{19A160C2-6897-43F9-AB25-0B60E506490B}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4827,7 +4852,7 @@
           <xm:sqref>G71</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="17" operator="equal" id="{C198F442-0CED-465D-B844-BD476FA91AED}">
+          <x14:cfRule type="cellIs" priority="19" operator="equal" id="{C198F442-0CED-465D-B844-BD476FA91AED}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4840,7 +4865,7 @@
           <xm:sqref>G76:G84</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="15" operator="equal" id="{B78ED6C4-4FF5-4C26-8AB0-814AD0D37A32}">
+          <x14:cfRule type="cellIs" priority="17" operator="equal" id="{B78ED6C4-4FF5-4C26-8AB0-814AD0D37A32}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4853,7 +4878,7 @@
           <xm:sqref>G86:G87</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="13" operator="equal" id="{5241F369-7025-4EA1-9AA0-9B9DA72E1877}">
+          <x14:cfRule type="cellIs" priority="15" operator="equal" id="{5241F369-7025-4EA1-9AA0-9B9DA72E1877}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4864,6 +4889,33 @@
             </x14:dxf>
           </x14:cfRule>
           <xm:sqref>G89</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{92DA3367-8274-43B1-9D44-4835DCEB0E0B}">
+            <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,G91)))</xm:f>
+            <xm:f>Restrictions!$B$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B0F0"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>G91:G92</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{BC362F27-3F33-4955-B3E6-521CFD463846}">
+            <xm:f>Restrictions!$B$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B0F0"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>G91:G92</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -4873,7 +4925,7 @@
           <x14:formula1>
             <xm:f>Restrictions!$A$1:$D$1</xm:f>
           </x14:formula1>
-          <xm:sqref>E1:E4 E6:E8 E10:E14 E16:E18 E20:E21 E109:E1048576 E27:E29 E23:E25 E103:E107 E31:E39 E41:E42 E44 E46:E51 E71:E74 E53:E55 E60:E63 E57:E58 E65:E69 E76:E84 E86:E89 E97:E101 E91:E95</xm:sqref>
+          <xm:sqref>E1:E4 E6:E8 E10:E14 E16:E18 E20:E21 E106:E1048576 E27:E29 E23:E25 E100:E104 E31:E39 E41:E42 E44 E46:E51 E71:E74 E53:E55 E60:E63 E57:E58 E65:E69 E76:E84 E86:E89 E94:E98 E91:E92</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4906,26 +4958,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a1b10758-7132-46a4-a2fe-7a2cf46f51f4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="f7d9f5a6-831d-4621-8c77-cbcaf993e406" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005A5B8F5EAAC22C48A11F5D9A60E6F21D" ma:contentTypeVersion="16" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="f2b963976306cc54294b7f4545a3c6c4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1b10758-7132-46a4-a2fe-7a2cf46f51f4" xmlns:ns3="f7d9f5a6-831d-4621-8c77-cbcaf993e406" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e5e135fa2fc1295e1586ddcd9c1a8904" ns2:_="" ns3:_="">
     <xsd:import namespace="a1b10758-7132-46a4-a2fe-7a2cf46f51f4"/>
@@ -5168,10 +5200,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a1b10758-7132-46a4-a2fe-7a2cf46f51f4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="f7d9f5a6-831d-4621-8c77-cbcaf993e406" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{40597E6F-FA73-4A07-893F-099FDC15B64D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="a1b10758-7132-46a4-a2fe-7a2cf46f51f4"/>
+    <ds:schemaRef ds:uri="f7d9f5a6-831d-4621-8c77-cbcaf993e406"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -5188,20 +5251,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{40597E6F-FA73-4A07-893F-099FDC15B64D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="a1b10758-7132-46a4-a2fe-7a2cf46f51f4"/>
-    <ds:schemaRef ds:uri="f7d9f5a6-831d-4621-8c77-cbcaf993e406"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix(Game): Finally got rid of the lag
The game is finally playable
</commit_message>
<xml_diff>
--- a/T_CraftMeUp_NeoDarbellay.xlsx
+++ b/T_CraftMeUp_NeoDarbellay.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01Modules\02Deuxieme_Annee\P_Prod\CraftMeUp\Craft-Me-Up\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1561886-3A06-49C1-84E4-F67D31D00C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E301384-46BD-49B1-BEBF-2CD2C6DFECB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
     <sheet name="Restrictions" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$G$106</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$G$97</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="158">
   <si>
     <t>Experts </t>
   </si>
@@ -430,9 +430,6 @@
     <t>Working on the biomes</t>
   </si>
   <si>
-    <t>S. Oliveira, G. Bianco and G Charmier</t>
-  </si>
-  <si>
     <t>Fixing an issue with camera clamping causing an error</t>
   </si>
   <si>
@@ -488,9 +485,6 @@
   </si>
   <si>
     <t>Day 19</t>
-  </si>
-  <si>
-    <t>Day 20</t>
   </si>
   <si>
     <t>Reduced rendering lag as much as I could for today
@@ -507,6 +501,21 @@
   </si>
   <si>
     <t>Tried to get rid of "TextHelpers", but it ended up creating more issues than anything. Next step is to cache</t>
+  </si>
+  <si>
+    <t>I noticed that there were issues with obstacle collisions, as there was no way to get nearby obstacles, so everything looped through every obstacle</t>
+  </si>
+  <si>
+    <t>Final rendering optimization</t>
+  </si>
+  <si>
+    <t>I believe the game is finally V2-Ready</t>
+  </si>
+  <si>
+    <t>S. Oliveira, G. Bianco and A. Gugler</t>
+  </si>
+  <si>
+    <t>Final memory optimization and V2 release</t>
   </si>
 </sst>
 </file>
@@ -729,7 +738,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -804,10 +813,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="22" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="20" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -837,10 +842,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -877,12 +878,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="85">
+  <dxfs count="84">
     <dxf>
       <fill>
         <patternFill>
@@ -1194,7 +1199,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B0F0"/>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1208,6 +1213,20 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
@@ -1215,6 +1234,27 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -1222,6 +1262,20 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -1229,6 +1283,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
@@ -1236,6 +1297,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -1243,6 +1311,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -1257,6 +1332,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -1264,6 +1346,20 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -1278,6 +1374,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -1285,6 +1388,20 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -1292,6 +1409,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
@@ -1299,6 +1423,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -1306,6 +1437,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -1313,161 +1451,21 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1788,7 +1786,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G108"/>
+  <dimension ref="A1:G99"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -1806,65 +1804,65 @@
       <c r="A1" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="37" t="s">
+      <c r="B1" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="38"/>
-      <c r="D1" s="35" t="s">
+      <c r="C1" s="36"/>
+      <c r="D1" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="E1" s="36"/>
-      <c r="F1" s="33" t="s">
+      <c r="E1" s="34"/>
+      <c r="F1" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="34"/>
+      <c r="G1" s="32"/>
     </row>
     <row r="2" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="38"/>
-      <c r="D2" s="35" t="s">
+      <c r="C2" s="36"/>
+      <c r="D2" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="36"/>
-      <c r="F2" s="33" t="s">
+      <c r="E2" s="34"/>
+      <c r="F2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="34"/>
+      <c r="G2" s="32"/>
     </row>
     <row r="3" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="B3" s="39" t="s">
-        <v>129</v>
-      </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="35" t="s">
+      <c r="B3" s="37" t="s">
+        <v>156</v>
+      </c>
+      <c r="C3" s="38"/>
+      <c r="D3" s="33" t="s">
         <v>87</v>
       </c>
-      <c r="E3" s="36"/>
-      <c r="F3" s="37" t="s">
+      <c r="E3" s="34"/>
+      <c r="F3" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="38"/>
+      <c r="G3" s="36"/>
     </row>
     <row r="4" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="43"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="43"/>
-      <c r="F4" s="43"/>
-      <c r="G4" s="38"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="36"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1873,7 +1871,7 @@
       <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="26" t="s">
         <v>89</v>
       </c>
       <c r="D5" s="2" t="s">
@@ -1893,7 +1891,7 @@
       <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="28">
+      <c r="B6" s="27">
         <v>45964</v>
       </c>
       <c r="C6" s="5">
@@ -1905,10 +1903,10 @@
       <c r="E6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="23">
+      <c r="F6" s="22">
         <v>0.59027777777777779</v>
       </c>
-      <c r="G6" s="24" t="s">
+      <c r="G6" s="23" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1916,7 +1914,7 @@
       <c r="A7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="29"/>
+      <c r="B7" s="28"/>
       <c r="C7" s="7">
         <v>35</v>
       </c>
@@ -1926,7 +1924,7 @@
       <c r="E7" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="23">
+      <c r="F7" s="22">
         <v>0.61458333333333337</v>
       </c>
       <c r="G7" s="19"/>
@@ -1935,7 +1933,7 @@
       <c r="A8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="29"/>
+      <c r="B8" s="28"/>
       <c r="C8" s="7">
         <v>60</v>
       </c>
@@ -1945,7 +1943,7 @@
       <c r="E8" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="23">
+      <c r="F8" s="22">
         <v>0.65625</v>
       </c>
       <c r="G8" s="8" t="s">
@@ -1962,19 +1960,19 @@
       <c r="C9" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D9" s="41">
+      <c r="D9" s="39">
         <f>SUM(C6:C8)</f>
         <v>125</v>
       </c>
-      <c r="E9" s="41"/>
-      <c r="F9" s="41"/>
-      <c r="G9" s="42"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
+      <c r="G9" s="40"/>
     </row>
     <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="28">
+      <c r="B10" s="27">
         <v>45965</v>
       </c>
       <c r="C10" s="5">
@@ -1986,7 +1984,7 @@
       <c r="E10" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="23">
+      <c r="F10" s="22">
         <v>0.36458333333333331</v>
       </c>
       <c r="G10" s="19"/>
@@ -1995,7 +1993,7 @@
       <c r="A11" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="29"/>
+      <c r="B11" s="28"/>
       <c r="C11" s="7">
         <v>50</v>
       </c>
@@ -2005,7 +2003,7 @@
       <c r="E11" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F11" s="23">
+      <c r="F11" s="22">
         <v>0.39930555555555558</v>
       </c>
       <c r="G11" s="8" t="s">
@@ -2016,7 +2014,7 @@
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="29"/>
+      <c r="B12" s="28"/>
       <c r="C12" s="7">
         <v>25</v>
       </c>
@@ -2026,7 +2024,7 @@
       <c r="E12" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F12" s="23">
+      <c r="F12" s="22">
         <v>0.42708333333333331</v>
       </c>
       <c r="G12" s="8" t="s">
@@ -2037,7 +2035,7 @@
       <c r="A13" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="29"/>
+      <c r="B13" s="28"/>
       <c r="C13" s="7">
         <v>35</v>
       </c>
@@ -2047,7 +2045,7 @@
       <c r="E13" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F13" s="23">
+      <c r="F13" s="22">
         <v>0.4513888888888889</v>
       </c>
       <c r="G13" s="19"/>
@@ -2056,7 +2054,7 @@
       <c r="A14" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="32"/>
+      <c r="B14" s="42"/>
       <c r="C14" s="9">
         <v>35</v>
       </c>
@@ -2066,7 +2064,7 @@
       <c r="E14" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F14" s="23">
+      <c r="F14" s="22">
         <v>0.47569444444444442</v>
       </c>
       <c r="G14" s="8" t="s">
@@ -2083,19 +2081,19 @@
       <c r="C15" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D15" s="41">
+      <c r="D15" s="39">
         <f>SUM(C10:C14)</f>
         <v>175</v>
       </c>
-      <c r="E15" s="41"/>
-      <c r="F15" s="41"/>
-      <c r="G15" s="42"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="40"/>
     </row>
     <row r="16" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="28">
+      <c r="B16" s="27">
         <v>45971</v>
       </c>
       <c r="C16" s="5">
@@ -2107,7 +2105,7 @@
       <c r="E16" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F16" s="23">
+      <c r="F16" s="22">
         <v>0.57986111111111105</v>
       </c>
       <c r="G16" s="8" t="s">
@@ -2118,7 +2116,7 @@
       <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B17" s="29"/>
+      <c r="B17" s="28"/>
       <c r="C17" s="7">
         <v>55</v>
       </c>
@@ -2128,7 +2126,7 @@
       <c r="E17" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F17" s="25">
+      <c r="F17" s="24">
         <v>0.63194444444444442</v>
       </c>
       <c r="G17" s="8" t="s">
@@ -2139,7 +2137,7 @@
       <c r="A18" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="29"/>
+      <c r="B18" s="28"/>
       <c r="C18" s="7">
         <v>45</v>
       </c>
@@ -2149,7 +2147,7 @@
       <c r="E18" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F18" s="23">
+      <c r="F18" s="22">
         <v>0.66319444444444442</v>
       </c>
       <c r="G18" s="8" t="s">
@@ -2166,19 +2164,19 @@
       <c r="C19" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D19" s="41">
+      <c r="D19" s="39">
         <f>SUM(C16:C18)</f>
         <v>145</v>
       </c>
-      <c r="E19" s="41"/>
-      <c r="F19" s="41"/>
-      <c r="G19" s="42"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="40"/>
     </row>
     <row r="20" spans="1:7" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="28">
+      <c r="B20" s="27">
         <v>45972</v>
       </c>
       <c r="C20" s="5"/>
@@ -2188,7 +2186,7 @@
       <c r="E20" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F20" s="23">
+      <c r="F20" s="22">
         <v>0.3923611111111111</v>
       </c>
       <c r="G20" s="8" t="s">
@@ -2199,7 +2197,7 @@
       <c r="A21" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="29"/>
+      <c r="B21" s="28"/>
       <c r="C21" s="7">
         <v>105</v>
       </c>
@@ -2209,7 +2207,7 @@
       <c r="E21" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F21" s="25">
+      <c r="F21" s="24">
         <v>0.47569444444444442</v>
       </c>
       <c r="G21" s="8" t="s">
@@ -2226,19 +2224,19 @@
       <c r="C22" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D22" s="41">
+      <c r="D22" s="39">
         <f>SUM(C20:C21)</f>
         <v>105</v>
       </c>
-      <c r="E22" s="41"/>
-      <c r="F22" s="41"/>
-      <c r="G22" s="42"/>
+      <c r="E22" s="39"/>
+      <c r="F22" s="39"/>
+      <c r="G22" s="40"/>
     </row>
     <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="28">
+      <c r="B23" s="27">
         <v>45978</v>
       </c>
       <c r="C23" s="5">
@@ -2250,7 +2248,7 @@
       <c r="E23" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F23" s="23">
+      <c r="F23" s="22">
         <v>0.63194444444444442</v>
       </c>
       <c r="G23" s="8" t="s">
@@ -2261,7 +2259,7 @@
       <c r="A24" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="29"/>
+      <c r="B24" s="28"/>
       <c r="C24" s="7">
         <v>10</v>
       </c>
@@ -2271,7 +2269,7 @@
       <c r="E24" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F24" s="23">
+      <c r="F24" s="22">
         <v>0.63888888888888895</v>
       </c>
       <c r="G24" s="19"/>
@@ -2280,7 +2278,7 @@
       <c r="A25" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="29"/>
+      <c r="B25" s="28"/>
       <c r="C25" s="9">
         <v>25</v>
       </c>
@@ -2290,7 +2288,7 @@
       <c r="E25" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F25" s="23">
+      <c r="F25" s="22">
         <v>0.65625</v>
       </c>
       <c r="G25" s="8" t="s">
@@ -2307,19 +2305,19 @@
       <c r="C26" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D26" s="41">
+      <c r="D26" s="39">
         <f>SUM(C23:C25)</f>
         <v>140</v>
       </c>
-      <c r="E26" s="41"/>
-      <c r="F26" s="41"/>
-      <c r="G26" s="42"/>
+      <c r="E26" s="39"/>
+      <c r="F26" s="39"/>
+      <c r="G26" s="40"/>
     </row>
     <row r="27" spans="1:7" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="28">
+      <c r="B27" s="27">
         <v>45979</v>
       </c>
       <c r="C27" s="5">
@@ -2331,7 +2329,7 @@
       <c r="E27" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F27" s="23">
+      <c r="F27" s="22">
         <v>0.4375</v>
       </c>
       <c r="G27" s="8" t="s">
@@ -2342,7 +2340,7 @@
       <c r="A28" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="29"/>
+      <c r="B28" s="28"/>
       <c r="C28" s="7">
         <v>45</v>
       </c>
@@ -2352,7 +2350,7 @@
       <c r="E28" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F28" s="23">
+      <c r="F28" s="22">
         <v>0.46875</v>
       </c>
       <c r="G28" s="8" t="s">
@@ -2363,7 +2361,7 @@
       <c r="A29" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="29"/>
+      <c r="B29" s="28"/>
       <c r="C29" s="7">
         <v>10</v>
       </c>
@@ -2373,7 +2371,7 @@
       <c r="E29" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F29" s="23">
+      <c r="F29" s="22">
         <v>0.47569444444444442</v>
       </c>
       <c r="G29" s="19"/>
@@ -2388,19 +2386,19 @@
       <c r="C30" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D30" s="41">
+      <c r="D30" s="39">
         <f>SUM(C27:C29)</f>
         <v>155</v>
       </c>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="42"/>
+      <c r="E30" s="39"/>
+      <c r="F30" s="39"/>
+      <c r="G30" s="40"/>
     </row>
     <row r="31" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B31" s="28">
+      <c r="B31" s="27">
         <v>45985</v>
       </c>
       <c r="C31" s="5">
@@ -2412,7 +2410,7 @@
       <c r="E31" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F31" s="23">
+      <c r="F31" s="22">
         <v>0.55555555555555558</v>
       </c>
       <c r="G31" s="19"/>
@@ -2421,7 +2419,7 @@
       <c r="A32" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B32" s="29"/>
+      <c r="B32" s="28"/>
       <c r="C32" s="7">
         <v>20</v>
       </c>
@@ -2431,7 +2429,7 @@
       <c r="E32" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F32" s="23">
+      <c r="F32" s="22">
         <v>0.56944444444444442</v>
       </c>
       <c r="G32" s="8" t="s">
@@ -2442,7 +2440,7 @@
       <c r="A33" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B33" s="29"/>
+      <c r="B33" s="28"/>
       <c r="C33" s="7">
         <v>30</v>
       </c>
@@ -2452,7 +2450,7 @@
       <c r="E33" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F33" s="23">
+      <c r="F33" s="22">
         <v>0.59027777777777779</v>
       </c>
       <c r="G33" s="19"/>
@@ -2461,7 +2459,7 @@
       <c r="A34" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B34" s="29"/>
+      <c r="B34" s="28"/>
       <c r="C34" s="7">
         <v>15</v>
       </c>
@@ -2471,7 +2469,7 @@
       <c r="E34" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F34" s="23">
+      <c r="F34" s="22">
         <v>0.60069444444444442</v>
       </c>
       <c r="G34" s="19"/>
@@ -2480,7 +2478,7 @@
       <c r="A35" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B35" s="29"/>
+      <c r="B35" s="28"/>
       <c r="C35" s="7">
         <v>10</v>
       </c>
@@ -2490,7 +2488,7 @@
       <c r="E35" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F35" s="23">
+      <c r="F35" s="22">
         <v>0.60763888888888895</v>
       </c>
       <c r="G35" s="19"/>
@@ -2499,7 +2497,7 @@
       <c r="A36" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B36" s="29"/>
+      <c r="B36" s="28"/>
       <c r="C36" s="7">
         <v>10</v>
       </c>
@@ -2509,7 +2507,7 @@
       <c r="E36" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F36" s="23">
+      <c r="F36" s="22">
         <v>0.61458333333333337</v>
       </c>
       <c r="G36" s="19"/>
@@ -2518,7 +2516,7 @@
       <c r="A37" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B37" s="29"/>
+      <c r="B37" s="28"/>
       <c r="C37" s="7">
         <v>30</v>
       </c>
@@ -2528,7 +2526,7 @@
       <c r="E37" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F37" s="23">
+      <c r="F37" s="22">
         <v>0.64583333333333337</v>
       </c>
       <c r="G37" s="19"/>
@@ -2537,7 +2535,7 @@
       <c r="A38" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B38" s="29"/>
+      <c r="B38" s="28"/>
       <c r="C38" s="7">
         <v>5</v>
       </c>
@@ -2547,7 +2545,7 @@
       <c r="E38" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F38" s="23">
+      <c r="F38" s="22">
         <v>0.64930555555555558</v>
       </c>
       <c r="G38" s="19"/>
@@ -2556,7 +2554,7 @@
       <c r="A39" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B39" s="29"/>
+      <c r="B39" s="28"/>
       <c r="C39" s="7">
         <v>10</v>
       </c>
@@ -2566,7 +2564,7 @@
       <c r="E39" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F39" s="23">
+      <c r="F39" s="22">
         <v>0.65625</v>
       </c>
       <c r="G39" s="8" t="s">
@@ -2583,19 +2581,19 @@
       <c r="C40" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D40" s="41">
+      <c r="D40" s="39">
         <f>SUM(C31:C39)</f>
         <v>140</v>
       </c>
-      <c r="E40" s="41"/>
-      <c r="F40" s="41"/>
-      <c r="G40" s="42"/>
+      <c r="E40" s="39"/>
+      <c r="F40" s="39"/>
+      <c r="G40" s="40"/>
     </row>
     <row r="41" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B41" s="28">
+      <c r="B41" s="27">
         <v>45986</v>
       </c>
       <c r="C41" s="5">
@@ -2607,7 +2605,7 @@
       <c r="E41" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F41" s="23">
+      <c r="F41" s="22">
         <v>0.34375</v>
       </c>
       <c r="G41" s="19"/>
@@ -2616,7 +2614,7 @@
       <c r="A42" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B42" s="29"/>
+      <c r="B42" s="28"/>
       <c r="C42" s="7">
         <v>175</v>
       </c>
@@ -2626,7 +2624,7 @@
       <c r="E42" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F42" s="25">
+      <c r="F42" s="24">
         <v>0.47569444444444442</v>
       </c>
       <c r="G42" s="8" t="s">
@@ -2643,19 +2641,19 @@
       <c r="C43" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D43" s="41">
+      <c r="D43" s="39">
         <f>SUM(C41:C42)</f>
         <v>190</v>
       </c>
-      <c r="E43" s="41"/>
-      <c r="F43" s="41"/>
-      <c r="G43" s="42"/>
+      <c r="E43" s="39"/>
+      <c r="F43" s="39"/>
+      <c r="G43" s="40"/>
     </row>
     <row r="44" spans="1:7" ht="48.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B44" s="26">
+      <c r="B44" s="25">
         <v>45992</v>
       </c>
       <c r="C44" s="5">
@@ -2667,7 +2665,7 @@
       <c r="E44" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F44" s="23">
+      <c r="F44" s="22">
         <v>0.65625</v>
       </c>
       <c r="G44" s="8" t="s">
@@ -2684,19 +2682,19 @@
       <c r="C45" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D45" s="41">
+      <c r="D45" s="39">
         <f>SUM(C44:C44)</f>
         <v>140</v>
       </c>
-      <c r="E45" s="41"/>
-      <c r="F45" s="41"/>
-      <c r="G45" s="42"/>
+      <c r="E45" s="39"/>
+      <c r="F45" s="39"/>
+      <c r="G45" s="40"/>
     </row>
     <row r="46" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B46" s="28">
+      <c r="B46" s="27">
         <v>45993</v>
       </c>
       <c r="C46" s="5">
@@ -2708,7 +2706,7 @@
       <c r="E46" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F46" s="23">
+      <c r="F46" s="22">
         <v>0.36458333333333331</v>
       </c>
       <c r="G46" s="19"/>
@@ -2717,7 +2715,7 @@
       <c r="A47" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="B47" s="29"/>
+      <c r="B47" s="28"/>
       <c r="C47" s="7">
         <v>75</v>
       </c>
@@ -2727,7 +2725,7 @@
       <c r="E47" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F47" s="23">
+      <c r="F47" s="22">
         <v>0.42708333333333331</v>
       </c>
       <c r="G47" s="19"/>
@@ -2736,7 +2734,7 @@
       <c r="A48" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B48" s="29"/>
+      <c r="B48" s="28"/>
       <c r="C48" s="7">
         <v>15</v>
       </c>
@@ -2746,7 +2744,7 @@
       <c r="E48" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F48" s="23">
+      <c r="F48" s="22">
         <v>0.4375</v>
       </c>
       <c r="G48" s="19"/>
@@ -2755,7 +2753,7 @@
       <c r="A49" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B49" s="29"/>
+      <c r="B49" s="28"/>
       <c r="C49" s="7">
         <v>10</v>
       </c>
@@ -2765,7 +2763,7 @@
       <c r="E49" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F49" s="23">
+      <c r="F49" s="22">
         <v>0.44444444444444442</v>
       </c>
       <c r="G49" s="19"/>
@@ -2774,7 +2772,7 @@
       <c r="A50" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B50" s="29"/>
+      <c r="B50" s="28"/>
       <c r="C50" s="7">
         <v>10</v>
       </c>
@@ -2784,7 +2782,7 @@
       <c r="E50" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F50" s="23">
+      <c r="F50" s="22">
         <v>0.4513888888888889</v>
       </c>
       <c r="G50" s="19"/>
@@ -2793,7 +2791,7 @@
       <c r="A51" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B51" s="29"/>
+      <c r="B51" s="28"/>
       <c r="C51" s="7">
         <v>35</v>
       </c>
@@ -2803,7 +2801,7 @@
       <c r="E51" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F51" s="23">
+      <c r="F51" s="22">
         <v>0.47569444444444442</v>
       </c>
       <c r="G51" s="19"/>
@@ -2818,19 +2816,19 @@
       <c r="C52" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D52" s="41">
+      <c r="D52" s="39">
         <f>SUM(C46:C51)</f>
         <v>190</v>
       </c>
-      <c r="E52" s="41"/>
-      <c r="F52" s="41"/>
-      <c r="G52" s="42"/>
+      <c r="E52" s="39"/>
+      <c r="F52" s="39"/>
+      <c r="G52" s="40"/>
     </row>
     <row r="53" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B53" s="28">
+      <c r="B53" s="27">
         <v>45999</v>
       </c>
       <c r="C53" s="5">
@@ -2842,7 +2840,7 @@
       <c r="E53" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F53" s="23">
+      <c r="F53" s="22">
         <v>0.375</v>
       </c>
       <c r="G53" s="8" t="s">
@@ -2853,7 +2851,7 @@
       <c r="A54" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B54" s="29"/>
+      <c r="B54" s="28"/>
       <c r="C54" s="7">
         <v>15</v>
       </c>
@@ -2863,7 +2861,7 @@
       <c r="E54" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F54" s="23">
+      <c r="F54" s="22">
         <v>0.38541666666666669</v>
       </c>
       <c r="G54" s="19"/>
@@ -2872,7 +2870,7 @@
       <c r="A55" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B55" s="29"/>
+      <c r="B55" s="28"/>
       <c r="C55" s="7">
         <v>65</v>
       </c>
@@ -2882,7 +2880,7 @@
       <c r="E55" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F55" s="23">
+      <c r="F55" s="22">
         <v>0.44097222222222227</v>
       </c>
       <c r="G55" s="8" t="s">
@@ -2899,19 +2897,19 @@
       <c r="C56" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D56" s="41">
+      <c r="D56" s="39">
         <f>SUM(C53:C55)</f>
         <v>140</v>
       </c>
-      <c r="E56" s="41"/>
-      <c r="F56" s="41"/>
-      <c r="G56" s="42"/>
+      <c r="E56" s="39"/>
+      <c r="F56" s="39"/>
+      <c r="G56" s="40"/>
     </row>
     <row r="57" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B57" s="28">
+      <c r="B57" s="27">
         <v>46006</v>
       </c>
       <c r="C57" s="5">
@@ -2923,7 +2921,7 @@
       <c r="E57" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F57" s="23">
+      <c r="F57" s="22">
         <v>0.55902777777777779</v>
       </c>
       <c r="G57" s="8" t="s">
@@ -2934,7 +2932,7 @@
       <c r="A58" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B58" s="29"/>
+      <c r="B58" s="28"/>
       <c r="C58" s="7">
         <v>125</v>
       </c>
@@ -2944,7 +2942,7 @@
       <c r="E58" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F58" s="23">
+      <c r="F58" s="22">
         <v>0.65625</v>
       </c>
       <c r="G58" s="8" t="s">
@@ -2961,19 +2959,19 @@
       <c r="C59" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D59" s="41">
+      <c r="D59" s="39">
         <f>SUM(C57:C58)</f>
         <v>140</v>
       </c>
-      <c r="E59" s="41"/>
-      <c r="F59" s="41"/>
-      <c r="G59" s="42"/>
+      <c r="E59" s="39"/>
+      <c r="F59" s="39"/>
+      <c r="G59" s="40"/>
     </row>
     <row r="60" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B60" s="28">
+      <c r="B60" s="27">
         <v>46007</v>
       </c>
       <c r="C60" s="5">
@@ -2985,7 +2983,7 @@
       <c r="E60" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F60" s="23">
+      <c r="F60" s="22">
         <v>0.375</v>
       </c>
       <c r="G60" s="8" t="s">
@@ -2996,7 +2994,7 @@
       <c r="A61" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B61" s="29"/>
+      <c r="B61" s="28"/>
       <c r="C61" s="7">
         <v>10</v>
       </c>
@@ -3006,7 +3004,7 @@
       <c r="E61" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F61" s="23">
+      <c r="F61" s="22">
         <v>0.38194444444444442</v>
       </c>
       <c r="G61" s="19"/>
@@ -3015,7 +3013,7 @@
       <c r="A62" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B62" s="29"/>
+      <c r="B62" s="28"/>
       <c r="C62" s="7">
         <v>45</v>
       </c>
@@ -3025,7 +3023,7 @@
       <c r="E62" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F62" s="23">
+      <c r="F62" s="22">
         <v>0.4236111111111111</v>
       </c>
       <c r="G62" s="19"/>
@@ -3034,7 +3032,7 @@
       <c r="A63" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B63" s="29"/>
+      <c r="B63" s="28"/>
       <c r="C63" s="7">
         <v>65</v>
       </c>
@@ -3044,7 +3042,7 @@
       <c r="E63" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F63" s="23">
+      <c r="F63" s="22">
         <v>0.47569444444444442</v>
       </c>
       <c r="G63" s="8" t="s">
@@ -3061,19 +3059,19 @@
       <c r="C64" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D64" s="41">
+      <c r="D64" s="39">
         <f>SUM(C60:C63)</f>
         <v>180</v>
       </c>
-      <c r="E64" s="41"/>
-      <c r="F64" s="41"/>
-      <c r="G64" s="42"/>
+      <c r="E64" s="39"/>
+      <c r="F64" s="39"/>
+      <c r="G64" s="40"/>
     </row>
     <row r="65" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B65" s="28">
+      <c r="B65" s="27">
         <v>46027</v>
       </c>
       <c r="C65" s="5">
@@ -3085,7 +3083,7 @@
       <c r="E65" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F65" s="23">
+      <c r="F65" s="22">
         <v>0.55208333333333337</v>
       </c>
       <c r="G65" s="19"/>
@@ -3094,7 +3092,7 @@
       <c r="A66" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B66" s="29"/>
+      <c r="B66" s="28"/>
       <c r="C66" s="7">
         <v>10</v>
       </c>
@@ -3104,7 +3102,7 @@
       <c r="E66" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F66" s="23">
+      <c r="F66" s="22">
         <v>0.55902777777777779</v>
       </c>
       <c r="G66" s="19"/>
@@ -3113,7 +3111,7 @@
       <c r="A67" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B67" s="29"/>
+      <c r="B67" s="28"/>
       <c r="C67" s="7">
         <v>10</v>
       </c>
@@ -3123,7 +3121,7 @@
       <c r="E67" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F67" s="23">
+      <c r="F67" s="22">
         <v>0.56597222222222221</v>
       </c>
       <c r="G67" s="19"/>
@@ -3132,7 +3130,7 @@
       <c r="A68" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B68" s="29"/>
+      <c r="B68" s="28"/>
       <c r="C68" s="7">
         <v>45</v>
       </c>
@@ -3142,7 +3140,7 @@
       <c r="E68" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F68" s="23">
+      <c r="F68" s="22">
         <v>0.59722222222222221</v>
       </c>
       <c r="G68" s="19"/>
@@ -3151,7 +3149,7 @@
       <c r="A69" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B69" s="29"/>
+      <c r="B69" s="28"/>
       <c r="C69" s="7">
         <v>70</v>
       </c>
@@ -3161,7 +3159,7 @@
       <c r="E69" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F69" s="23">
+      <c r="F69" s="22">
         <v>0.65625</v>
       </c>
       <c r="G69" s="19" t="s">
@@ -3178,19 +3176,19 @@
       <c r="C70" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D70" s="41">
+      <c r="D70" s="39">
         <f>SUM(C65:C69)</f>
         <v>145</v>
       </c>
-      <c r="E70" s="41"/>
-      <c r="F70" s="41"/>
-      <c r="G70" s="42"/>
+      <c r="E70" s="39"/>
+      <c r="F70" s="39"/>
+      <c r="G70" s="40"/>
     </row>
     <row r="71" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B71" s="28">
+      <c r="B71" s="27">
         <v>46042</v>
       </c>
       <c r="C71" s="5">
@@ -3202,7 +3200,7 @@
       <c r="E71" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F71" s="23">
+      <c r="F71" s="22">
         <v>0.4375</v>
       </c>
       <c r="G71" s="8" t="s">
@@ -3213,7 +3211,7 @@
       <c r="A72" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B72" s="29"/>
+      <c r="B72" s="28"/>
       <c r="C72" s="7">
         <v>5</v>
       </c>
@@ -3223,7 +3221,7 @@
       <c r="E72" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F72" s="23">
+      <c r="F72" s="22">
         <v>0.44097222222222227</v>
       </c>
       <c r="G72" s="19"/>
@@ -3232,7 +3230,7 @@
       <c r="A73" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B73" s="29"/>
+      <c r="B73" s="28"/>
       <c r="C73" s="7">
         <v>40</v>
       </c>
@@ -3242,7 +3240,7 @@
       <c r="E73" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F73" s="23">
+      <c r="F73" s="22">
         <v>0.46527777777777773</v>
       </c>
       <c r="G73" s="19"/>
@@ -3251,7 +3249,7 @@
       <c r="A74" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B74" s="29"/>
+      <c r="B74" s="28"/>
       <c r="C74" s="7">
         <v>15</v>
       </c>
@@ -3261,7 +3259,7 @@
       <c r="E74" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F74" s="23">
+      <c r="F74" s="22">
         <v>0.47569444444444442</v>
       </c>
       <c r="G74" s="19"/>
@@ -3276,19 +3274,19 @@
       <c r="C75" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D75" s="41">
+      <c r="D75" s="39">
         <f>SUM(C71:C74)</f>
         <v>195</v>
       </c>
-      <c r="E75" s="41"/>
-      <c r="F75" s="41"/>
-      <c r="G75" s="42"/>
+      <c r="E75" s="39"/>
+      <c r="F75" s="39"/>
+      <c r="G75" s="40"/>
     </row>
     <row r="76" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B76" s="28">
+      <c r="B76" s="27">
         <v>46049</v>
       </c>
       <c r="C76" s="7">
@@ -3300,7 +3298,7 @@
       <c r="E76" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F76" s="23">
+      <c r="F76" s="22">
         <v>0.34375</v>
       </c>
       <c r="G76" s="8"/>
@@ -3309,38 +3307,38 @@
       <c r="A77" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B77" s="29"/>
+      <c r="B77" s="28"/>
       <c r="C77" s="7">
         <v>25</v>
       </c>
       <c r="D77" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E77" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F77" s="22">
+        <v>0.36458333333333331</v>
+      </c>
+      <c r="G77" s="8" t="s">
         <v>130</v>
-      </c>
-      <c r="E77" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F77" s="23">
-        <v>0.36458333333333331</v>
-      </c>
-      <c r="G77" s="8" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B78" s="29"/>
+      <c r="B78" s="28"/>
       <c r="C78" s="7">
         <v>10</v>
       </c>
       <c r="D78" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E78" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F78" s="23">
+      <c r="F78" s="22">
         <v>0.37152777777777773</v>
       </c>
       <c r="G78" s="8"/>
@@ -3349,38 +3347,38 @@
       <c r="A79" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B79" s="29"/>
+      <c r="B79" s="28"/>
       <c r="C79" s="7">
         <v>65</v>
       </c>
       <c r="D79" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E79" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F79" s="23">
+      <c r="F79" s="22">
         <v>0.42708333333333331</v>
       </c>
       <c r="G79" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B80" s="29"/>
+      <c r="B80" s="28"/>
       <c r="C80" s="7">
         <v>15</v>
       </c>
       <c r="D80" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E80" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F80" s="23">
+      <c r="F80" s="22">
         <v>0.4375</v>
       </c>
       <c r="G80" s="8"/>
@@ -3389,17 +3387,17 @@
       <c r="A81" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B81" s="29"/>
+      <c r="B81" s="28"/>
       <c r="C81" s="7">
         <v>40</v>
       </c>
       <c r="D81" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E81" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F81" s="23">
+      <c r="F81" s="22">
         <v>0.46527777777777773</v>
       </c>
       <c r="G81" s="8"/>
@@ -3408,17 +3406,17 @@
       <c r="A82" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B82" s="29"/>
+      <c r="B82" s="28"/>
       <c r="C82" s="7">
         <v>15</v>
       </c>
       <c r="D82" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E82" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F82" s="23">
+      <c r="F82" s="22">
         <v>0.47569444444444442</v>
       </c>
       <c r="G82" s="8"/>
@@ -3427,38 +3425,38 @@
       <c r="A83" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B83" s="29"/>
+      <c r="B83" s="28"/>
       <c r="C83" s="7">
         <v>25</v>
       </c>
       <c r="D83" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="E83" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F83" s="22">
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="G83" s="8" t="s">
         <v>139</v>
-      </c>
-      <c r="E83" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F83" s="23">
-        <v>0.61458333333333337</v>
-      </c>
-      <c r="G83" s="8" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="84" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B84" s="32"/>
+      <c r="B84" s="42"/>
       <c r="C84" s="7">
         <v>5</v>
       </c>
       <c r="D84" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E84" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F84" s="23">
+      <c r="F84" s="22">
         <v>0.63888888888888895</v>
       </c>
       <c r="G84" s="8"/>
@@ -3473,52 +3471,52 @@
       <c r="C85" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D85" s="41">
+      <c r="D85" s="39">
         <f>SUM(C76:C84)</f>
         <v>215</v>
       </c>
-      <c r="E85" s="41"/>
-      <c r="F85" s="41"/>
-      <c r="G85" s="42"/>
+      <c r="E85" s="39"/>
+      <c r="F85" s="39"/>
+      <c r="G85" s="40"/>
     </row>
     <row r="86" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B86" s="28">
+      <c r="B86" s="27">
         <v>46063</v>
       </c>
       <c r="C86" s="5">
         <v>10</v>
       </c>
       <c r="D86" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F86" s="22">
+        <v>0.34027777777777773</v>
+      </c>
+      <c r="G86" s="8" t="s">
         <v>143</v>
-      </c>
-      <c r="E86" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F86" s="23">
-        <v>0.34027777777777773</v>
-      </c>
-      <c r="G86" s="8" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B87" s="29"/>
+      <c r="B87" s="28"/>
       <c r="C87" s="7">
         <v>55</v>
       </c>
       <c r="D87" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E87" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F87" s="23">
+      <c r="F87" s="22">
         <v>0.37847222222222227</v>
       </c>
       <c r="G87" s="8"/>
@@ -3527,17 +3525,17 @@
       <c r="A88" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B88" s="29"/>
+      <c r="B88" s="28"/>
       <c r="C88" s="7">
         <v>40</v>
       </c>
       <c r="D88" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E88" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F88" s="23">
+      <c r="F88" s="22">
         <v>0.41666666666666669</v>
       </c>
       <c r="G88" s="19"/>
@@ -3546,21 +3544,21 @@
       <c r="A89" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B89" s="29"/>
+      <c r="B89" s="28"/>
       <c r="C89" s="7">
         <v>85</v>
       </c>
       <c r="D89" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E89" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F89" s="23">
+      <c r="F89" s="22">
         <v>0.47569444444444442</v>
       </c>
       <c r="G89" s="8" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="90" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -3568,61 +3566,61 @@
         <v>95</v>
       </c>
       <c r="B90" s="17" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C90" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D90" s="41">
+      <c r="D90" s="39">
         <f>SUM(C86:C89)</f>
         <v>190</v>
       </c>
-      <c r="E90" s="41"/>
-      <c r="F90" s="41"/>
-      <c r="G90" s="42"/>
+      <c r="E90" s="39"/>
+      <c r="F90" s="39"/>
+      <c r="G90" s="40"/>
     </row>
     <row r="91" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B91" s="28">
+      <c r="B91" s="27">
         <v>46084</v>
       </c>
       <c r="C91" s="5">
         <v>105</v>
       </c>
       <c r="D91" s="8" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E91" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F91" s="23">
+      <c r="F91" s="22">
         <v>0.41666666666666669</v>
       </c>
       <c r="G91" s="8" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B92" s="29"/>
+      <c r="B92" s="28"/>
       <c r="C92" s="7">
         <v>85</v>
       </c>
       <c r="D92" s="8" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E92" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F92" s="23">
+      <c r="F92" s="22">
         <v>0.47569444444444442</v>
       </c>
       <c r="G92" s="8" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -3630,173 +3628,111 @@
         <v>95</v>
       </c>
       <c r="B93" s="17" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C93" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D93" s="41">
+      <c r="D93" s="39">
         <f>SUM(C91:C92)</f>
         <v>190</v>
       </c>
-      <c r="E93" s="41"/>
-      <c r="F93" s="41"/>
-      <c r="G93" s="42"/>
-    </row>
-    <row r="94" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="4"/>
-      <c r="B94" s="28"/>
-      <c r="C94" s="5"/>
-      <c r="D94" s="8"/>
-      <c r="E94" s="8"/>
-      <c r="F94" s="22"/>
-      <c r="G94" s="19"/>
-    </row>
-    <row r="95" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="6"/>
-      <c r="B95" s="29"/>
-      <c r="C95" s="7"/>
-      <c r="D95" s="8"/>
-      <c r="E95" s="8"/>
-      <c r="F95" s="22"/>
-      <c r="G95" s="19"/>
-    </row>
-    <row r="96" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="6"/>
-      <c r="B96" s="29"/>
-      <c r="C96" s="7"/>
-      <c r="D96" s="8"/>
-      <c r="E96" s="8"/>
-      <c r="F96" s="7"/>
-      <c r="G96" s="19"/>
-    </row>
-    <row r="97" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="6"/>
-      <c r="B97" s="29"/>
-      <c r="C97" s="7"/>
-      <c r="D97" s="8"/>
-      <c r="E97" s="8"/>
-      <c r="F97" s="7"/>
-      <c r="G97" s="19"/>
-    </row>
-    <row r="98" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="9"/>
-      <c r="B98" s="32"/>
-      <c r="C98" s="9"/>
-      <c r="D98" s="8"/>
-      <c r="E98" s="10"/>
-      <c r="F98" s="7"/>
-      <c r="G98" s="19"/>
-    </row>
-    <row r="99" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="11" t="s">
+      <c r="E93" s="39"/>
+      <c r="F93" s="39"/>
+      <c r="G93" s="40"/>
+    </row>
+    <row r="94" spans="1:7" ht="72" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B94" s="27">
+        <v>46098</v>
+      </c>
+      <c r="C94" s="5">
+        <v>55</v>
+      </c>
+      <c r="D94" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="E94" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F94" s="22">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="G94" s="8" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B95" s="28"/>
+      <c r="C95" s="7">
+        <v>35</v>
+      </c>
+      <c r="D95" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="E95" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F95" s="22">
+        <v>0.44097222222222227</v>
+      </c>
+      <c r="G95" s="8" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="B99" s="17" t="s">
-        <v>148</v>
-      </c>
-      <c r="C99" s="17" t="s">
+      <c r="B96" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="C96" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D99" s="41">
-        <f>SUM(C94:C98)</f>
-        <v>0</v>
-      </c>
-      <c r="E99" s="41"/>
-      <c r="F99" s="41"/>
-      <c r="G99" s="42"/>
-    </row>
-    <row r="100" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="4"/>
-      <c r="B100" s="28"/>
-      <c r="C100" s="5"/>
-      <c r="D100" s="8"/>
-      <c r="E100" s="8"/>
-      <c r="F100" s="22"/>
-      <c r="G100" s="19"/>
-    </row>
-    <row r="101" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A101" s="6"/>
-      <c r="B101" s="29"/>
-      <c r="C101" s="7"/>
-      <c r="D101" s="8"/>
-      <c r="E101" s="8"/>
-      <c r="F101" s="22"/>
-      <c r="G101" s="19"/>
-    </row>
-    <row r="102" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="6"/>
-      <c r="B102" s="29"/>
-      <c r="C102" s="7"/>
-      <c r="D102" s="8"/>
-      <c r="E102" s="8"/>
-      <c r="F102" s="7"/>
-      <c r="G102" s="19"/>
-    </row>
-    <row r="103" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="6"/>
-      <c r="B103" s="29"/>
-      <c r="C103" s="7"/>
-      <c r="D103" s="8"/>
-      <c r="E103" s="8"/>
-      <c r="F103" s="7"/>
-      <c r="G103" s="19"/>
-    </row>
-    <row r="104" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A104" s="9"/>
-      <c r="B104" s="32"/>
-      <c r="C104" s="9"/>
-      <c r="D104" s="8"/>
-      <c r="E104" s="10"/>
-      <c r="F104" s="7"/>
-      <c r="G104" s="19"/>
-    </row>
-    <row r="105" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A105" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="B105" s="17" t="s">
-        <v>149</v>
-      </c>
-      <c r="C105" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="D105" s="41">
-        <f>SUM(C100:C104)</f>
-        <v>0</v>
-      </c>
-      <c r="E105" s="41"/>
-      <c r="F105" s="41"/>
-      <c r="G105" s="42"/>
-    </row>
-    <row r="106" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A106" s="30" t="s">
+      <c r="D96" s="39">
+        <f>SUM(C94:C95)</f>
+        <v>90</v>
+      </c>
+      <c r="E96" s="39"/>
+      <c r="F96" s="39"/>
+      <c r="G96" s="40"/>
+    </row>
+    <row r="97" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="29" t="s">
         <v>111</v>
       </c>
-      <c r="B106" s="31"/>
-      <c r="C106" s="12">
-        <f>MROUND(SUM(C6:C105) /60,0.2)</f>
-        <v>48.400000000000006</v>
-      </c>
-      <c r="D106" s="13"/>
-      <c r="E106" s="18"/>
-      <c r="F106" s="20"/>
-      <c r="G106" s="14"/>
-    </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A107" s="15"/>
-    </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A108" s="15"/>
+      <c r="B97" s="30"/>
+      <c r="C97" s="12">
+        <f>MROUND(SUM(C6:C96) /60,0.2)</f>
+        <v>49.800000000000004</v>
+      </c>
+      <c r="D97" s="13"/>
+      <c r="E97" s="18"/>
+      <c r="F97" s="20"/>
+      <c r="G97" s="14"/>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A98" s="15"/>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A99" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="50">
+  <mergeCells count="48">
+    <mergeCell ref="D85:G85"/>
+    <mergeCell ref="D90:G90"/>
+    <mergeCell ref="D96:G96"/>
+    <mergeCell ref="D93:G93"/>
     <mergeCell ref="D22:G22"/>
     <mergeCell ref="D26:G26"/>
     <mergeCell ref="D30:G30"/>
     <mergeCell ref="D40:G40"/>
-    <mergeCell ref="B76:B84"/>
-    <mergeCell ref="D105:G105"/>
     <mergeCell ref="D52:G52"/>
     <mergeCell ref="D43:G43"/>
     <mergeCell ref="D45:G45"/>
@@ -3805,10 +3741,6 @@
     <mergeCell ref="D56:G56"/>
     <mergeCell ref="D59:G59"/>
     <mergeCell ref="D64:G64"/>
-    <mergeCell ref="D85:G85"/>
-    <mergeCell ref="D90:G90"/>
-    <mergeCell ref="D99:G99"/>
-    <mergeCell ref="D93:G93"/>
     <mergeCell ref="D9:G9"/>
     <mergeCell ref="D15:G15"/>
     <mergeCell ref="D19:G19"/>
@@ -3828,9 +3760,8 @@
     <mergeCell ref="B20:B21"/>
     <mergeCell ref="B23:B25"/>
     <mergeCell ref="B27:B29"/>
-    <mergeCell ref="A106:B106"/>
+    <mergeCell ref="A97:B97"/>
     <mergeCell ref="B31:B39"/>
-    <mergeCell ref="B100:B104"/>
     <mergeCell ref="B46:B51"/>
     <mergeCell ref="B41:B42"/>
     <mergeCell ref="B71:B74"/>
@@ -3839,15 +3770,16 @@
     <mergeCell ref="B57:B58"/>
     <mergeCell ref="B60:B63"/>
     <mergeCell ref="B86:B89"/>
-    <mergeCell ref="B94:B98"/>
+    <mergeCell ref="B94:B95"/>
     <mergeCell ref="B91:B92"/>
+    <mergeCell ref="B76:B84"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C100:C104 C27:C29 C23:C25 C16:C18 B6 C10:C14 C20:C21 C6:C8 C31:C39 C41:C42 C44 C46:C51 C71:C74 C53:C55 C60:C63 C57:C58 C65:C69 C76:C84 C86:C89 C94:C98 C91:C92" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C27:C29 C23:C25 C16:C18 B6 C10:C14 C20:C21 C6:C8 C31:C39 C41:C42 C44 C46:C51 C71:C74 C53:C55 C60:C63 C57:C58 C65:C69 C76:C84 C86:C89 C94:C95 C91:C92" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B10:B14 B16:B18 B20:B21 B100:B104 B27:B29 B23:B25 B31:B39 B41:B42 B44 B46:B51 B71:B74 B53:B55 B60:B63 B57:B58 B65:B69 B76 B86:B89 B94:B98 B91:B92" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B10:B14 B16:B18 B20:B21 B27:B29 B23:B25 B31:B39 B41:B42 B44 B46:B51 B71:B74 B53:B55 B60:B63 B57:B58 B65:B69 B76 B86:B89 B94:B95 B91:B92" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -3857,7 +3789,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="28" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" scale="29" orientation="portrait" r:id="rId3"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -3867,7 +3799,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="111" operator="equal" id="{6BC2577B-BDA3-4B48-8F95-0F2177F9264F}">
+          <x14:cfRule type="cellIs" priority="113" operator="equal" id="{6BC2577B-BDA3-4B48-8F95-0F2177F9264F}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3877,10 +3809,20 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>A4:E8 A10:E14 A16:E18 A20:E21 A23:E25 A27:E29 A31:E39 A100:E104 A106:E1048576 A44:E44 A41:E42 A46:E51 A71:E74 A65:E69 A60:E63 A57:E58 A53:E55 A86:E89 A76:E76 C77:E84 A94:E98 A91:E92 A1:D2 F1:F3 A3 D3 G4:G5 G7:G8 A9:D9 A15:D15 A19:D19 A22:D22 A26:D26 A30:D30 A40:D40 A43:D43 A45:D45 A52:D52 A56:D56 A59:D59 A64:D64 A70:D70 A75:D75 A77:A84 A85:D85 A90:D90 A93:D93 A99:D99 A105:D105 G106:G1048576</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="110" operator="equal" id="{9C6C644F-7238-453A-BC69-B42FAB3A2FA5}">
+          <xm:sqref>A4:E8 A10:E14 A16:E18 A20:E21 A23:E25 A27:E29 A31:E39 A97:E1048576 A44:E44 A41:E42 A46:E51 A71:E74 A65:E69 A60:E63 A57:E58 A53:E55 A86:E89 A76:E76 C77:E84 A94:E95 A91:E92 A1:D2 F1:F3 A3 D3 G4:G5 G7:G8 A9:D9 A15:D15 A19:D19 A22:D22 A26:D26 A30:D30 A40:D40 A43:D43 A45:D45 A52:D52 A56:D56 A59:D59 A64:D64 A70:D70 A75:D75 A77:A84 A85:D85 A90:D90 A93:D93 A96:D96 G97:G1048576</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="114" operator="equal" id="{6DE85145-1CAE-407F-B647-4C9B303613C7}">
+            <xm:f>Restrictions!$C$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="112" operator="equal" id="{9C6C644F-7238-453A-BC69-B42FAB3A2FA5}">
             <xm:f>Restrictions!$A$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3890,7 +3832,30 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="112" operator="equal" id="{6DE85145-1CAE-407F-B647-4C9B303613C7}">
+          <x14:cfRule type="cellIs" priority="115" operator="equal" id="{29EA468D-F98D-4D41-AA55-B63DA0941363}">
+            <xm:f>Restrictions!$D$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>E4:E8 E10:E14 E16:E18 E20:E21 E23:E25 E27:E29 E31:E39 E97:E1048576</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="83" operator="equal" id="{DA16BC0E-098E-492D-9DD4-7AE32F5A0B66}">
+            <xm:f>Restrictions!$D$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="82" operator="equal" id="{B6903E1B-29F5-497F-B030-3589B8B337A1}">
             <xm:f>Restrictions!$C$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3900,7 +3865,20 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="113" operator="equal" id="{29EA468D-F98D-4D41-AA55-B63DA0941363}">
+          <x14:cfRule type="cellIs" priority="81" operator="equal" id="{84E995EC-6FB3-447D-B7B4-F39F6B4AAF45}">
+            <xm:f>Restrictions!$A$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B050"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>E41:E42</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="87" operator="equal" id="{FFFCA022-7518-426F-AC53-14AA2D86A5EB}">
             <xm:f>Restrictions!$D$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3910,10 +3888,17 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E4:E8 E10:E14 E16:E18 E20:E21 E23:E25 E27:E29 E31:E39 E100:E104 E106:E1048576</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="79" operator="equal" id="{84E995EC-6FB3-447D-B7B4-F39F6B4AAF45}">
+          <x14:cfRule type="cellIs" priority="86" operator="equal" id="{29283CD5-B4A3-4A92-85FA-0825B9BB0F20}">
+            <xm:f>Restrictions!$C$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="85" operator="equal" id="{2763426F-5E05-4AE5-BAB9-6155B44E42F3}">
             <xm:f>Restrictions!$A$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3923,7 +3908,20 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="80" operator="equal" id="{B6903E1B-29F5-497F-B030-3589B8B337A1}">
+          <xm:sqref>E44</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="75" operator="equal" id="{7CBCFDCF-397F-4B71-B6B1-D6B8B3D995CF}">
+            <xm:f>Restrictions!$D$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="74" operator="equal" id="{8AA9BDE2-93E5-4C8F-8ABB-C8A37EF6C1F7}">
             <xm:f>Restrictions!$C$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3933,7 +3931,30 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="81" operator="equal" id="{DA16BC0E-098E-492D-9DD4-7AE32F5A0B66}">
+          <x14:cfRule type="cellIs" priority="73" operator="equal" id="{55BA1703-E0F0-4534-AC5F-5524C52012B8}">
+            <xm:f>Restrictions!$A$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B050"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>E46:E51</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="53" operator="equal" id="{38CC099F-2CFB-4F51-BCC6-9A8C062F12D6}">
+            <xm:f>Restrictions!$A$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B050"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="55" operator="equal" id="{9BE9A0C0-12EE-4A06-AA91-2B2C7773C591}">
             <xm:f>Restrictions!$D$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3943,10 +3964,40 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E41:E42</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="83" operator="equal" id="{2763426F-5E05-4AE5-BAB9-6155B44E42F3}">
+          <x14:cfRule type="cellIs" priority="54" operator="equal" id="{97B7369B-F3E2-421C-8B11-B917735F9E01}">
+            <xm:f>Restrictions!$C$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>E53:E55</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="59" operator="equal" id="{06F1F730-9D3E-44F6-9858-23332EAE481C}">
+            <xm:f>Restrictions!$D$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="58" operator="equal" id="{E33B63BE-9C2D-46FB-840B-160E77C144D1}">
+            <xm:f>Restrictions!$C$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="57" operator="equal" id="{CE91AE07-0A4B-4CA1-864E-4494D1FD3F2D}">
             <xm:f>Restrictions!$A$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3956,7 +4007,30 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="84" operator="equal" id="{29283CD5-B4A3-4A92-85FA-0825B9BB0F20}">
+          <xm:sqref>E57:E58</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="61" operator="equal" id="{6138D6EC-9477-4522-A720-100D44F804C5}">
+            <xm:f>Restrictions!$A$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B050"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="63" operator="equal" id="{F3D48842-32E0-470D-8962-C942EB8B670B}">
+            <xm:f>Restrictions!$D$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="62" operator="equal" id="{7FB697E4-A1F6-44CC-8422-CFE46191EC29}">
             <xm:f>Restrictions!$C$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3966,7 +4040,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="85" operator="equal" id="{FFFCA022-7518-426F-AC53-14AA2D86A5EB}">
+          <xm:sqref>E60:E63</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="67" operator="equal" id="{806E81D0-33D7-43D5-9F66-9ACF5303AA2B}">
             <xm:f>Restrictions!$D$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3976,10 +4053,17 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E44</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="71" operator="equal" id="{55BA1703-E0F0-4534-AC5F-5524C52012B8}">
+          <x14:cfRule type="cellIs" priority="66" operator="equal" id="{5A6DBF38-AB31-41CF-92EB-6F71330B8A51}">
+            <xm:f>Restrictions!$C$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="65" operator="equal" id="{CF4E2A7B-2831-4A8E-8CB0-05A3819B6512}">
             <xm:f>Restrictions!$A$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3989,7 +4073,20 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="72" operator="equal" id="{8AA9BDE2-93E5-4C8F-8ABB-C8A37EF6C1F7}">
+          <xm:sqref>E65:E69</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="71" operator="equal" id="{5E85ED66-7E81-44BB-AFFF-3FBE898F7448}">
+            <xm:f>Restrictions!$D$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="70" operator="equal" id="{CCF6CA8D-69A5-48BE-8938-2E3B52B06A90}">
             <xm:f>Restrictions!$C$1</xm:f>
             <x14:dxf>
               <fill>
@@ -3999,7 +4096,20 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="73" operator="equal" id="{7CBCFDCF-397F-4B71-B6B1-D6B8B3D995CF}">
+          <x14:cfRule type="cellIs" priority="69" operator="equal" id="{EC003FB1-6A08-40D6-88B1-588BCE936C35}">
+            <xm:f>Restrictions!$A$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B050"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>E71:E74</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="24" operator="equal" id="{5EE1483C-C8AF-4BC8-96C2-1FBDBB50C066}">
             <xm:f>Restrictions!$D$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4009,10 +4119,17 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E46:E51</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="51" operator="equal" id="{38CC099F-2CFB-4F51-BCC6-9A8C062F12D6}">
+          <x14:cfRule type="cellIs" priority="23" operator="equal" id="{CAD63670-76D8-46C3-9428-FF1328E16D90}">
+            <xm:f>Restrictions!$C$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="22" operator="equal" id="{42B27148-AE7C-4BA1-B993-B3037B69F92A}">
             <xm:f>Restrictions!$A$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4022,7 +4139,30 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="52" operator="equal" id="{97B7369B-F3E2-421C-8B11-B917735F9E01}">
+          <xm:sqref>E76:E84</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="27" operator="equal" id="{8A959092-8A6B-4A91-99D1-8110E43AA729}">
+            <xm:f>Restrictions!$A$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B050"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="29" operator="equal" id="{8CF84F96-ED65-491E-B676-DA2F761CE9EB}">
+            <xm:f>Restrictions!$D$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="28" operator="equal" id="{F801D24C-AFDA-4757-9BC6-FB24B4DE466D}">
             <xm:f>Restrictions!$C$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4032,7 +4172,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="53" operator="equal" id="{9BE9A0C0-12EE-4A06-AA91-2B2C7773C591}">
+          <xm:sqref>E86:E89</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{5CAB61E4-56FF-4285-A4C9-A33737017E3A}">
             <xm:f>Restrictions!$D$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4042,10 +4185,17 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E53:E55</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="55" operator="equal" id="{CE91AE07-0A4B-4CA1-864E-4494D1FD3F2D}">
+          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{9E114EAB-BD08-4433-A88A-51FDBB871F00}">
+            <xm:f>Restrictions!$C$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{92E62023-F404-4026-AD69-5B76EB0BDAE8}">
             <xm:f>Restrictions!$A$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4055,7 +4205,30 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="56" operator="equal" id="{E33B63BE-9C2D-46FB-840B-160E77C144D1}">
+          <xm:sqref>E91:E92</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="10" operator="equal" id="{A66F7540-0CD1-4EF9-B347-2CABE04E932F}">
+            <xm:f>Restrictions!$A$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B050"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{59C9B578-9F2D-494D-BED9-807E89EADAB8}">
+            <xm:f>Restrictions!$D$1</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="11" operator="equal" id="{E10A4C2F-1FA6-426F-A318-4C7EFBFBAD06}">
             <xm:f>Restrictions!$C$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4065,251 +4238,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="57" operator="equal" id="{06F1F730-9D3E-44F6-9858-23332EAE481C}">
-            <xm:f>Restrictions!$D$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFF0000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>E57:E58</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="59" operator="equal" id="{6138D6EC-9477-4522-A720-100D44F804C5}">
-            <xm:f>Restrictions!$A$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B050"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="60" operator="equal" id="{7FB697E4-A1F6-44CC-8422-CFE46191EC29}">
-            <xm:f>Restrictions!$C$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFC000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="61" operator="equal" id="{F3D48842-32E0-470D-8962-C942EB8B670B}">
-            <xm:f>Restrictions!$D$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFF0000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>E60:E63</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="63" operator="equal" id="{CF4E2A7B-2831-4A8E-8CB0-05A3819B6512}">
-            <xm:f>Restrictions!$A$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B050"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="64" operator="equal" id="{5A6DBF38-AB31-41CF-92EB-6F71330B8A51}">
-            <xm:f>Restrictions!$C$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFC000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="65" operator="equal" id="{806E81D0-33D7-43D5-9F66-9ACF5303AA2B}">
-            <xm:f>Restrictions!$D$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFF0000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>E65:E69</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="67" operator="equal" id="{EC003FB1-6A08-40D6-88B1-588BCE936C35}">
-            <xm:f>Restrictions!$A$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B050"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="68" operator="equal" id="{CCF6CA8D-69A5-48BE-8938-2E3B52B06A90}">
-            <xm:f>Restrictions!$C$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFC000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="69" operator="equal" id="{5E85ED66-7E81-44BB-AFFF-3FBE898F7448}">
-            <xm:f>Restrictions!$D$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFF0000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>E71:E74</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="20" operator="equal" id="{42B27148-AE7C-4BA1-B993-B3037B69F92A}">
-            <xm:f>Restrictions!$A$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B050"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="21" operator="equal" id="{CAD63670-76D8-46C3-9428-FF1328E16D90}">
-            <xm:f>Restrictions!$C$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFC000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="22" operator="equal" id="{5EE1483C-C8AF-4BC8-96C2-1FBDBB50C066}">
-            <xm:f>Restrictions!$D$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFF0000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>E76:E84</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="25" operator="equal" id="{8A959092-8A6B-4A91-99D1-8110E43AA729}">
-            <xm:f>Restrictions!$A$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B050"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="26" operator="equal" id="{F801D24C-AFDA-4757-9BC6-FB24B4DE466D}">
-            <xm:f>Restrictions!$C$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFC000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="27" operator="equal" id="{8CF84F96-ED65-491E-B676-DA2F761CE9EB}">
-            <xm:f>Restrictions!$D$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFF0000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>E86:E89</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{92E62023-F404-4026-AD69-5B76EB0BDAE8}">
-            <xm:f>Restrictions!$A$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B050"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{9E114EAB-BD08-4433-A88A-51FDBB871F00}">
-            <xm:f>Restrictions!$C$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFC000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{5CAB61E4-56FF-4285-A4C9-A33737017E3A}">
-            <xm:f>Restrictions!$D$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFF0000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>E91:E92</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{A66F7540-0CD1-4EF9-B347-2CABE04E932F}">
-            <xm:f>Restrictions!$A$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B050"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{E10A4C2F-1FA6-426F-A318-4C7EFBFBAD06}">
-            <xm:f>Restrictions!$C$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFC000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="10" operator="equal" id="{59C9B578-9F2D-494D-BED9-807E89EADAB8}">
-            <xm:f>Restrictions!$D$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFF0000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>E94:E98</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="107" operator="containsText" id="{FD0F452B-B2F8-4F75-A8CD-A69AC0834E64}">
+          <xm:sqref>E94:E95</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="109" operator="containsText" id="{FD0F452B-B2F8-4F75-A8CD-A69AC0834E64}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F6)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4323,7 +4255,7 @@
           <xm:sqref>F6:F8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="105" operator="containsText" id="{6407061A-B268-44CE-A52C-133739941B16}">
+          <x14:cfRule type="containsText" priority="107" operator="containsText" id="{6407061A-B268-44CE-A52C-133739941B16}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F16)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4337,7 +4269,7 @@
           <xm:sqref>F16:F18</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="104" operator="containsText" id="{756A584A-6AAC-4559-9F27-A59B4EFD7F34}">
+          <x14:cfRule type="containsText" priority="106" operator="containsText" id="{756A584A-6AAC-4559-9F27-A59B4EFD7F34}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F20)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4351,7 +4283,7 @@
           <xm:sqref>F20:F21</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="103" operator="containsText" id="{E988FD75-2909-4816-91C7-1018002A435D}">
+          <x14:cfRule type="containsText" priority="105" operator="containsText" id="{E988FD75-2909-4816-91C7-1018002A435D}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F23)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4365,7 +4297,7 @@
           <xm:sqref>F23 F24:G24 F25</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="102" operator="containsText" id="{D5B6D5DF-9E2A-4C4B-BA82-97D983766AEE}">
+          <x14:cfRule type="containsText" priority="104" operator="containsText" id="{D5B6D5DF-9E2A-4C4B-BA82-97D983766AEE}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F27)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4379,7 +4311,7 @@
           <xm:sqref>F27:F28 F29:G29</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="82" operator="containsText" id="{58D84678-3AF3-4F30-A017-BCF30ADC23B9}">
+          <x14:cfRule type="containsText" priority="84" operator="containsText" id="{58D84678-3AF3-4F30-A017-BCF30ADC23B9}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F44)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4393,7 +4325,7 @@
           <xm:sqref>F44</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="50" operator="containsText" id="{2CEED9A6-BF96-4A7D-A6A3-A1CBCB1BBB33}">
+          <x14:cfRule type="containsText" priority="52" operator="containsText" id="{2CEED9A6-BF96-4A7D-A6A3-A1CBCB1BBB33}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F53)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4407,7 +4339,7 @@
           <xm:sqref>F53 F54:G54 F55</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="54" operator="containsText" id="{9846E030-D336-4ABF-8549-0B217B1EE9C0}">
+          <x14:cfRule type="containsText" priority="56" operator="containsText" id="{9846E030-D336-4ABF-8549-0B217B1EE9C0}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F57)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4421,7 +4353,7 @@
           <xm:sqref>F57:F58</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="58" operator="containsText" id="{C331D7E9-51D1-4558-86A6-2DDD97E5F51B}">
+          <x14:cfRule type="containsText" priority="60" operator="containsText" id="{C331D7E9-51D1-4558-86A6-2DDD97E5F51B}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F60)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4435,7 +4367,7 @@
           <xm:sqref>F60 F61:G62 F63</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="66" operator="containsText" id="{A87BC3C4-539A-4D6D-94C0-DF4DFEA06C8A}">
+          <x14:cfRule type="containsText" priority="68" operator="containsText" id="{A87BC3C4-539A-4D6D-94C0-DF4DFEA06C8A}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F71)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4449,7 +4381,7 @@
           <xm:sqref>F71 F72:G74</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="23" operator="containsText" id="{94391AE6-F1AE-42D1-AF78-4812D68E41C4}">
+          <x14:cfRule type="containsText" priority="25" operator="containsText" id="{94391AE6-F1AE-42D1-AF78-4812D68E41C4}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F84)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4463,7 +4395,7 @@
           <xm:sqref>F84</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="106" operator="containsText" id="{88417B48-EA26-4D48-9EFE-B6A1E5C426AE}">
+          <x14:cfRule type="containsText" priority="108" operator="containsText" id="{88417B48-EA26-4D48-9EFE-B6A1E5C426AE}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F10)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4477,7 +4409,7 @@
           <xm:sqref>F10:G10 F11:F12 F13:G13 F14</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="101" operator="containsText" id="{1555D56B-E8B5-4F0A-9D80-B2C1016EB105}">
+          <x14:cfRule type="containsText" priority="103" operator="containsText" id="{1555D56B-E8B5-4F0A-9D80-B2C1016EB105}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F31)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4491,7 +4423,7 @@
           <xm:sqref>F31:G31 F32</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="90" operator="containsText" id="{F174B00B-9E6F-49FA-9EE7-95FA16CF0425}">
+          <x14:cfRule type="containsText" priority="92" operator="containsText" id="{F174B00B-9E6F-49FA-9EE7-95FA16CF0425}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F33)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4505,7 +4437,7 @@
           <xm:sqref>F33:G38 F39</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="78" operator="containsText" id="{4AF076A7-8EED-499A-B340-9301C9A23B63}">
+          <x14:cfRule type="containsText" priority="80" operator="containsText" id="{4AF076A7-8EED-499A-B340-9301C9A23B63}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F41)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4519,7 +4451,7 @@
           <xm:sqref>F41:G41 F42</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="70" operator="containsText" id="{1E89304F-1BDF-40FA-83E9-2770D86CCD7D}">
+          <x14:cfRule type="containsText" priority="72" operator="containsText" id="{1E89304F-1BDF-40FA-83E9-2770D86CCD7D}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F46)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4533,7 +4465,7 @@
           <xm:sqref>F46:G51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="62" operator="containsText" id="{FBCB4E68-F50D-4BE4-8CEE-A9CE7EAE06EE}">
+          <x14:cfRule type="containsText" priority="64" operator="containsText" id="{FBCB4E68-F50D-4BE4-8CEE-A9CE7EAE06EE}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F65)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4547,7 +4479,7 @@
           <xm:sqref>F65:G69</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="36" operator="containsText" id="{3688DB4D-873A-4169-BE4C-08434A027D62}">
+          <x14:cfRule type="containsText" priority="38" operator="containsText" id="{3688DB4D-873A-4169-BE4C-08434A027D62}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F76)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4561,7 +4493,7 @@
           <xm:sqref>F76:G76 F77 F78:G79 F80</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="29" operator="containsText" id="{1CA0FC1F-6CFD-462C-912C-B25E380596FE}">
+          <x14:cfRule type="containsText" priority="31" operator="containsText" id="{1CA0FC1F-6CFD-462C-912C-B25E380596FE}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F81)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4575,7 +4507,7 @@
           <xm:sqref>F81:G83</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="16" operator="containsText" id="{6EAE5B84-F778-418F-A1B7-BC9BA100112D}">
+          <x14:cfRule type="containsText" priority="18" operator="containsText" id="{6EAE5B84-F778-418F-A1B7-BC9BA100112D}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F86)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4589,7 +4521,7 @@
           <xm:sqref>F86:G89</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{49774D53-9CD8-4DDA-86D7-61DDC39694A2}">
+          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{92DA3367-8274-43B1-9D44-4835DCEB0E0B}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F91)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4600,10 +4532,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>F91:F92</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="7" operator="containsText" id="{EC18E800-531E-417C-9061-1973EA038CA3}">
+          <xm:sqref>F91:G92</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{F4DDEC4D-7298-464C-A521-1EDC13E32A16}">
             <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F94)))</xm:f>
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
@@ -4614,11 +4546,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>F94:G98</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="100" operator="containsText" id="{2F0F41F7-8C93-48A6-B013-C45F8E29AE34}">
-            <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,F100)))</xm:f>
+          <xm:sqref>F94:G95</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="101" operator="equal" id="{C81CB296-EBDE-4E68-996A-22E647E300C9}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4628,10 +4559,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>F100:G104</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="99" operator="equal" id="{C81CB296-EBDE-4E68-996A-22E647E300C9}">
+          <xm:sqref>G11:G12</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="100" operator="equal" id="{C6523CE4-984A-4BEA-B850-BBE212DEC1BD}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4641,10 +4572,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G11:G12</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="98" operator="equal" id="{C6523CE4-984A-4BEA-B850-BBE212DEC1BD}">
+          <xm:sqref>G14</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="99" operator="equal" id="{34CA0963-7227-4B81-A491-AF5EBF6948E0}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4654,10 +4585,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G14</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="97" operator="equal" id="{34CA0963-7227-4B81-A491-AF5EBF6948E0}">
+          <xm:sqref>G16:G18</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="98" operator="equal" id="{0137ED0B-0223-4A2D-BBA6-66B7E7B0177B}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4667,10 +4598,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G16:G18</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="96" operator="equal" id="{0137ED0B-0223-4A2D-BBA6-66B7E7B0177B}">
+          <xm:sqref>G20:G21</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="97" operator="equal" id="{0559BE0C-06E8-4BF0-855B-46B347A65A43}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4680,10 +4611,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G20:G21</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="95" operator="equal" id="{0559BE0C-06E8-4BF0-855B-46B347A65A43}">
+          <xm:sqref>G23</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="96" operator="equal" id="{A10A680C-18B8-4576-98EE-F30E41E55578}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4693,10 +4624,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G23</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="94" operator="equal" id="{A10A680C-18B8-4576-98EE-F30E41E55578}">
+          <xm:sqref>G25</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="95" operator="equal" id="{EE200D4C-87A3-41C0-AADC-DBA0F1BBC7B2}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4706,10 +4637,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G25</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="93" operator="equal" id="{EE200D4C-87A3-41C0-AADC-DBA0F1BBC7B2}">
+          <xm:sqref>G27:G28</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="94" operator="equal" id="{11814DC1-0D86-496F-AEC1-5E73F0134CB6}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4719,10 +4650,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G27:G28</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="92" operator="equal" id="{11814DC1-0D86-496F-AEC1-5E73F0134CB6}">
+          <xm:sqref>G32</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="79" operator="equal" id="{267A3B51-36A4-44DF-B2E6-F06E71682E5F}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4732,10 +4663,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G32</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="77" operator="equal" id="{267A3B51-36A4-44DF-B2E6-F06E71682E5F}">
+          <xm:sqref>G39</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="78" operator="equal" id="{0FA35E81-D3C4-44FE-9341-C74ABA01B1FF}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4745,10 +4676,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G39</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="76" operator="equal" id="{0FA35E81-D3C4-44FE-9341-C74ABA01B1FF}">
+          <xm:sqref>G42</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="77" operator="equal" id="{E1E75134-FA7A-4AB7-9C7B-BBBAB5BA6AE8}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4758,10 +4689,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G42</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="75" operator="equal" id="{E1E75134-FA7A-4AB7-9C7B-BBBAB5BA6AE8}">
+          <xm:sqref>G44</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="51" operator="equal" id="{7506C776-F73B-475A-A848-0E98C716D28F}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4771,10 +4702,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G44</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="49" operator="equal" id="{7506C776-F73B-475A-A848-0E98C716D28F}">
+          <xm:sqref>G53</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="50" operator="equal" id="{EEDBCFEE-8EE0-4370-A603-3DD0D0A3C004}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4784,10 +4715,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G53</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="48" operator="equal" id="{EEDBCFEE-8EE0-4370-A603-3DD0D0A3C004}">
+          <xm:sqref>G55</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="49" operator="equal" id="{EBD16DC6-D1FA-4FC5-B74B-CA3CF0413675}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4797,10 +4728,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G55</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="47" operator="equal" id="{EBD16DC6-D1FA-4FC5-B74B-CA3CF0413675}">
+          <xm:sqref>G57:G58</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="48" operator="equal" id="{CB5C53FD-3D5D-4030-A78E-D6ACDDA5D5F7}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4810,10 +4741,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G57:G58</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="46" operator="equal" id="{CB5C53FD-3D5D-4030-A78E-D6ACDDA5D5F7}">
+          <xm:sqref>G60</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="47" operator="equal" id="{28414CE1-4551-493E-98F2-E4708C3326DE}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4823,10 +4754,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G60</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="45" operator="equal" id="{28414CE1-4551-493E-98F2-E4708C3326DE}">
+          <xm:sqref>G63</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="46" operator="equal" id="{19A160C2-6897-43F9-AB25-0B60E506490B}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4836,10 +4767,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G63</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="44" operator="equal" id="{19A160C2-6897-43F9-AB25-0B60E506490B}">
+          <xm:sqref>G71</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="21" operator="equal" id="{C198F442-0CED-465D-B844-BD476FA91AED}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4849,10 +4780,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G71</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="19" operator="equal" id="{C198F442-0CED-465D-B844-BD476FA91AED}">
+          <xm:sqref>G76:G84</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="19" operator="equal" id="{B78ED6C4-4FF5-4C26-8AB0-814AD0D37A32}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4862,10 +4793,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G76:G84</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="17" operator="equal" id="{B78ED6C4-4FF5-4C26-8AB0-814AD0D37A32}">
+          <xm:sqref>G86:G87</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="17" operator="equal" id="{5241F369-7025-4EA1-9AA0-9B9DA72E1877}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4875,10 +4806,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G86:G87</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="15" operator="equal" id="{5241F369-7025-4EA1-9AA0-9B9DA72E1877}">
+          <xm:sqref>G89</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{BC362F27-3F33-4955-B3E6-521CFD463846}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4888,11 +4819,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G89</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{92DA3367-8274-43B1-9D44-4835DCEB0E0B}">
-            <xm:f>NOT(ISERROR(SEARCH(Restrictions!$B$1,G91)))</xm:f>
+          <xm:sqref>G91:G92</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{F36AC5F6-B024-4CC2-9E60-F561F2DD8C64}">
             <xm:f>Restrictions!$B$1</xm:f>
             <x14:dxf>
               <fill>
@@ -4902,20 +4832,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G91:G92</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{BC362F27-3F33-4955-B3E6-521CFD463846}">
-            <xm:f>Restrictions!$B$1</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B0F0"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>G91:G92</xm:sqref>
+          <xm:sqref>G94:G95</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -4925,7 +4842,7 @@
           <x14:formula1>
             <xm:f>Restrictions!$A$1:$D$1</xm:f>
           </x14:formula1>
-          <xm:sqref>E1:E4 E6:E8 E10:E14 E16:E18 E20:E21 E106:E1048576 E27:E29 E23:E25 E100:E104 E31:E39 E41:E42 E44 E46:E51 E71:E74 E53:E55 E60:E63 E57:E58 E65:E69 E76:E84 E86:E89 E94:E98 E91:E92</xm:sqref>
+          <xm:sqref>E1:E4 E6:E8 E10:E14 E16:E18 E20:E21 E97:E1048576 E27:E29 E23:E25 E31:E39 E41:E42 E44 E46:E51 E71:E74 E53:E55 E60:E63 E57:E58 E65:E69 E76:E84 E86:E89 E94:E95 E91:E92</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>